<commit_message>
adicionando 2 automatização para criar pasta (usar uma unica vez) e o outro puxa foto e converte para png
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1638c87186bceadf/Desktop/OfertasTec/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="11_F9695CA42DBBB00D7708F6DF240B1251B879C294" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B6D98F19-8F14-412B-AD16-EB05E3675314}"/>
+  <xr:revisionPtr revIDLastSave="53" documentId="11_F9695CA42DBBB00D7708F6DF240B1251B879C294" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AB0688C-7B48-48BA-BC41-00E7B9218022}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1792,7 +1792,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1873,29 +1873,13 @@
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC00000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -7499,19 +7483,19 @@
       <c r="E253" s="20"/>
     </row>
     <row r="254" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B254" s="29"/>
+      <c r="B254" s="58"/>
       <c r="E254" s="20"/>
     </row>
     <row r="255" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B255" s="29"/>
+      <c r="B255" s="58"/>
       <c r="E255" s="20"/>
     </row>
     <row r="256" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B256" s="29"/>
+      <c r="B256" s="58"/>
       <c r="E256" s="20"/>
     </row>
     <row r="257" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B257" s="29"/>
+      <c r="B257" s="58"/>
       <c r="E257" s="20"/>
     </row>
     <row r="258" spans="2:5" x14ac:dyDescent="0.25">
@@ -7636,6 +7620,7 @@
       <c r="E1974"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I253" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
criação de subpastas na pasta principal fotos-webp
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1638c87186bceadf/Desktop/OfertasTec/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_AAE99CEC2896977288487518AB0B1651B879BB5B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5C98F01-509B-46DF-A0FE-F6C415968AC0}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_AAE99CEC2896977288487518AB0B1651B879BB5B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B3FAF33-F3FF-4810-A5F4-7472D876727C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Produtos Renomear" sheetId="1" r:id="rId1"/>
@@ -1792,7 +1792,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1875,7 +1875,6 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -1892,6 +1891,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2179,6 +2182,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA1974"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2222,7 +2226,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
       <c r="B2" s="29">
         <v>1</v>
@@ -2245,7 +2249,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="29">
         <v>2</v>
@@ -2268,7 +2272,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="29">
         <v>3</v>
@@ -2291,7 +2295,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="55">
         <v>4</v>
@@ -2312,7 +2316,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
       <c r="B6" s="29">
         <v>5</v>
@@ -2335,7 +2339,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" s="29">
         <v>6</v>
@@ -2358,7 +2362,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="29">
         <v>7</v>
@@ -2381,7 +2385,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
       <c r="B9" s="29">
         <v>8</v>
@@ -2404,7 +2408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="29">
         <v>9</v>
@@ -2427,7 +2431,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="55">
         <v>10</v>
@@ -2452,7 +2456,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="29">
         <v>11</v>
@@ -2475,7 +2479,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="29">
         <v>12</v>
@@ -2498,7 +2502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="29">
         <v>13</v>
@@ -2521,7 +2525,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="29">
         <v>14</v>
@@ -2544,7 +2548,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="55">
         <v>15</v>
@@ -2567,7 +2571,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="56">
         <v>16</v>
@@ -2592,7 +2596,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="29">
         <v>17</v>
@@ -2615,7 +2619,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="29">
         <v>18</v>
@@ -2638,7 +2642,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="55">
         <v>19</v>
@@ -2657,7 +2661,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="29">
         <v>20</v>
@@ -2680,7 +2684,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="55">
         <v>21</v>
@@ -2699,7 +2703,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="29">
         <v>22</v>
@@ -2722,7 +2726,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="55">
         <v>23</v>
@@ -2745,7 +2749,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="55">
         <v>24</v>
@@ -2764,7 +2768,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="29">
         <v>25</v>
@@ -2787,7 +2791,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="29">
         <v>26</v>
@@ -2810,7 +2814,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="29">
         <v>27</v>
@@ -2833,7 +2837,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="47"/>
       <c r="B29" s="48">
         <v>28</v>
@@ -2856,7 +2860,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="29">
         <v>29</v>
@@ -2879,7 +2883,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="29">
         <v>30</v>
@@ -2902,7 +2906,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="56">
         <v>31</v>
@@ -2927,7 +2931,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="55">
         <v>32</v>
@@ -2950,7 +2954,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="29">
         <v>33</v>
@@ -2973,7 +2977,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="47"/>
       <c r="B35" s="48">
         <v>34</v>
@@ -2996,7 +3000,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="29">
         <v>35</v>
@@ -3019,7 +3023,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="29">
         <v>36</v>
@@ -3042,7 +3046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="29">
         <v>37</v>
@@ -3065,7 +3069,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="29">
         <v>38</v>
@@ -3088,7 +3092,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
       <c r="B40" s="29">
         <v>39</v>
@@ -3111,7 +3115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="29">
         <v>40</v>
@@ -3134,7 +3138,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="55">
         <v>41</v>
@@ -3153,7 +3157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
       <c r="B43" s="29">
         <v>42</v>
@@ -3176,7 +3180,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="55">
         <v>43</v>
@@ -3195,7 +3199,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
       <c r="B45" s="29">
         <v>44</v>
@@ -3218,7 +3222,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="29">
         <v>45</v>
@@ -3241,7 +3245,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="55">
         <v>46</v>
@@ -3264,7 +3268,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="29">
         <v>47</v>
@@ -3287,7 +3291,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="55">
         <v>48</v>
@@ -3306,7 +3310,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="29">
         <v>49</v>
@@ -3329,7 +3333,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
       <c r="B51" s="29">
         <v>50</v>
@@ -3352,7 +3356,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="29">
         <v>51</v>
@@ -3375,7 +3379,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="29">
         <v>52</v>
@@ -3398,7 +3402,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="29">
         <v>53</v>
@@ -3421,7 +3425,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="29">
         <v>54</v>
@@ -3444,7 +3448,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="29">
         <v>55</v>
@@ -3897,7 +3901,6 @@
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="60"/>
       <c r="B76" s="37">
         <v>75</v>
       </c>
@@ -4189,7 +4192,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="16"/>
       <c r="B89" s="29">
         <v>88</v>
@@ -4212,7 +4215,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="16"/>
       <c r="B90" s="29">
         <v>89</v>
@@ -4235,7 +4238,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="16"/>
       <c r="B91" s="29">
         <v>90</v>
@@ -4258,7 +4261,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="16"/>
       <c r="B92" s="29">
         <v>91</v>
@@ -4281,7 +4284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="55">
         <v>92</v>
@@ -4300,7 +4303,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="16"/>
       <c r="B94" s="29">
         <v>93</v>
@@ -4323,7 +4326,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="16"/>
       <c r="B95" s="29">
         <v>94</v>
@@ -4346,7 +4349,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="16"/>
       <c r="B96" s="29">
         <v>95</v>
@@ -4369,7 +4372,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="16"/>
       <c r="B97" s="29">
         <v>96</v>
@@ -4392,7 +4395,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="55">
         <v>97</v>
@@ -4411,7 +4414,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="55">
         <v>98</v>
@@ -4430,7 +4433,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="16"/>
       <c r="B100" s="29">
         <v>99</v>
@@ -4453,7 +4456,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="16"/>
       <c r="B101" s="29">
         <v>100</v>
@@ -4476,7 +4479,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="16"/>
       <c r="B102" s="29">
         <v>101</v>
@@ -4499,7 +4502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="55">
         <v>102</v>
@@ -4522,7 +4525,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="16"/>
       <c r="B104" s="29">
         <v>103</v>
@@ -4545,7 +4548,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="55">
         <v>104</v>
@@ -4564,7 +4567,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="16"/>
       <c r="B106" s="29">
         <v>105</v>
@@ -4587,7 +4590,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="16"/>
       <c r="B107" s="29">
         <v>106</v>
@@ -4610,7 +4613,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="16"/>
       <c r="B108" s="29">
         <v>107</v>
@@ -4633,7 +4636,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="55">
         <v>108</v>
@@ -4652,7 +4655,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="16"/>
       <c r="B110" s="29">
         <v>109</v>
@@ -4675,7 +4678,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="16"/>
       <c r="B111" s="29">
         <v>110</v>
@@ -4698,7 +4701,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="16"/>
       <c r="B112" s="29">
         <v>111</v>
@@ -4721,7 +4724,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="9"/>
       <c r="B113" s="56">
         <v>112</v>
@@ -4740,7 +4743,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="16"/>
       <c r="B114" s="29">
         <v>113</v>
@@ -4763,7 +4766,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="16"/>
       <c r="B115" s="29">
         <v>114</v>
@@ -4786,7 +4789,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="16"/>
       <c r="B116" s="29">
         <v>115</v>
@@ -4809,7 +4812,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="16"/>
       <c r="B117" s="29">
         <v>116</v>
@@ -4832,7 +4835,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3"/>
       <c r="B118" s="55">
         <v>117</v>
@@ -4851,7 +4854,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="16"/>
       <c r="B119" s="29">
         <v>118</v>
@@ -4874,7 +4877,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="16"/>
       <c r="B120" s="29">
         <v>119</v>
@@ -4897,7 +4900,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="16"/>
       <c r="B121" s="29">
         <v>120</v>
@@ -4920,7 +4923,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3"/>
       <c r="B122" s="55">
         <v>121</v>
@@ -4939,7 +4942,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="16"/>
       <c r="B123" s="29">
         <v>122</v>
@@ -4962,7 +4965,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="16"/>
       <c r="B124" s="29">
         <v>123</v>
@@ -4985,7 +4988,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="12"/>
       <c r="B125" s="29">
         <v>124</v>
@@ -5008,7 +5011,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="16"/>
       <c r="B126" s="29">
         <v>125</v>
@@ -5031,7 +5034,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="16"/>
       <c r="B127" s="29">
         <v>126</v>
@@ -5054,7 +5057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="16"/>
       <c r="B128" s="29">
         <v>127</v>
@@ -5077,7 +5080,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="16"/>
       <c r="B129" s="29">
         <v>128</v>
@@ -5100,7 +5103,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="16"/>
       <c r="B130" s="29">
         <v>129</v>
@@ -5123,7 +5126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="16"/>
       <c r="B131" s="29">
         <v>130</v>
@@ -5146,7 +5149,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="16"/>
       <c r="B132" s="29">
         <v>131</v>
@@ -5169,7 +5172,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="16"/>
       <c r="B133" s="29">
         <v>132</v>
@@ -5192,7 +5195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="16"/>
       <c r="B134" s="29">
         <v>133</v>
@@ -5215,7 +5218,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="16"/>
       <c r="B135" s="29">
         <v>134</v>
@@ -5238,7 +5241,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="16"/>
       <c r="B136" s="29">
         <v>135</v>
@@ -5261,7 +5264,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="16"/>
       <c r="B137" s="29">
         <v>136</v>
@@ -5284,7 +5287,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="16"/>
       <c r="B138" s="33">
         <v>137</v>
@@ -5309,7 +5312,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="16"/>
       <c r="B139" s="29">
         <v>138</v>
@@ -5332,7 +5335,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="16"/>
       <c r="B140" s="29">
         <v>139</v>
@@ -5355,7 +5358,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="141" spans="1:9" s="57" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" s="57" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="16"/>
       <c r="B141" s="29">
         <v>140</v>
@@ -5375,7 +5378,7 @@
       </c>
       <c r="H141" s="29"/>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="16"/>
       <c r="B142" s="29">
         <v>141</v>
@@ -5395,7 +5398,7 @@
       </c>
       <c r="H142" s="29"/>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="16"/>
       <c r="B143" s="29">
         <v>142</v>
@@ -5415,7 +5418,7 @@
       </c>
       <c r="H143" s="29"/>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="16"/>
       <c r="B144" s="29">
         <v>143</v>
@@ -5435,7 +5438,7 @@
       </c>
       <c r="H144" s="29"/>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="9"/>
       <c r="B145" s="56">
         <v>144</v>
@@ -5457,7 +5460,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="16"/>
       <c r="B146" s="29">
         <v>145</v>
@@ -5477,7 +5480,7 @@
       </c>
       <c r="H146" s="29"/>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="16"/>
       <c r="B147" s="29">
         <v>146</v>
@@ -5497,7 +5500,7 @@
       </c>
       <c r="H147" s="29"/>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="16"/>
       <c r="B148" s="29">
         <v>147</v>
@@ -5517,7 +5520,7 @@
       </c>
       <c r="H148" s="29"/>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="16"/>
       <c r="B149" s="29">
         <v>148</v>
@@ -5537,7 +5540,7 @@
       </c>
       <c r="H149" s="29"/>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="9"/>
       <c r="B150" s="56">
         <v>149</v>
@@ -5559,7 +5562,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="151" spans="1:9" s="47" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" s="47" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B151" s="48">
         <v>150</v>
       </c>
@@ -5578,7 +5581,7 @@
       </c>
       <c r="H151" s="48"/>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="16"/>
       <c r="B152" s="29">
         <v>151</v>
@@ -5598,7 +5601,7 @@
       </c>
       <c r="H152" s="29"/>
     </row>
-    <row r="153" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" ht="21.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="16"/>
       <c r="B153" s="29">
         <v>152</v>
@@ -5618,7 +5621,7 @@
       </c>
       <c r="H153" s="29"/>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="16"/>
       <c r="B154" s="29">
         <v>153</v>
@@ -5638,7 +5641,7 @@
       </c>
       <c r="H154" s="29"/>
     </row>
-    <row r="155" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" ht="21.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9"/>
       <c r="B155" s="56">
         <v>154</v>
@@ -5660,7 +5663,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="3"/>
       <c r="B156" s="55">
         <v>155</v>
@@ -5679,7 +5682,7 @@
       <c r="H156" s="3"/>
       <c r="I156" s="3"/>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="16"/>
       <c r="B157" s="29">
         <v>156</v>
@@ -5697,7 +5700,7 @@
       <c r="G157" s="29"/>
       <c r="H157" s="29"/>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B158" s="29">
         <v>157</v>
       </c>
@@ -5714,7 +5717,7 @@
       <c r="G158" s="29"/>
       <c r="H158" s="29"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B159" s="56">
         <v>158</v>
       </c>
@@ -5733,7 +5736,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B160" s="56">
         <v>159</v>
       </c>
@@ -5752,7 +5755,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="161" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B161" s="29">
         <v>160</v>
       </c>
@@ -5770,7 +5773,7 @@
       <c r="H161" s="31"/>
       <c r="I161" s="5"/>
     </row>
-    <row r="162" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B162" s="56">
         <v>161</v>
       </c>
@@ -5808,7 +5811,7 @@
       <c r="Z162" s="5"/>
       <c r="AA162" s="5"/>
     </row>
-    <row r="163" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
       <c r="B163" s="55">
         <v>162</v>
@@ -5845,7 +5848,7 @@
       <c r="Z163" s="5"/>
       <c r="AA163" s="5"/>
     </row>
-    <row r="164" spans="1:27" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:27" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="26"/>
       <c r="B164" s="56">
         <v>163</v>
@@ -5884,7 +5887,7 @@
       <c r="Z164" s="5"/>
       <c r="AA164" s="5"/>
     </row>
-    <row r="165" spans="1:27" s="26" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:27" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="B165" s="29">
         <v>164</v>
       </c>
@@ -5920,7 +5923,7 @@
       <c r="Z165" s="5"/>
       <c r="AA165" s="5"/>
     </row>
-    <row r="166" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B166" s="29">
         <v>165</v>
       </c>
@@ -5956,7 +5959,7 @@
       <c r="Z166" s="5"/>
       <c r="AA166" s="5"/>
     </row>
-    <row r="167" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B167" s="29">
         <v>166</v>
       </c>
@@ -5992,7 +5995,7 @@
       <c r="Z167" s="5"/>
       <c r="AA167" s="5"/>
     </row>
-    <row r="168" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B168" s="29">
         <v>167</v>
       </c>
@@ -6028,7 +6031,7 @@
       <c r="Z168" s="5"/>
       <c r="AA168" s="5"/>
     </row>
-    <row r="169" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B169" s="56">
         <v>168</v>
       </c>
@@ -6066,7 +6069,7 @@
       <c r="Z169" s="5"/>
       <c r="AA169" s="5"/>
     </row>
-    <row r="170" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B170" s="29">
         <v>169</v>
       </c>
@@ -6102,7 +6105,7 @@
       <c r="Z170" s="5"/>
       <c r="AA170" s="5"/>
     </row>
-    <row r="171" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B171" s="29">
         <v>170</v>
       </c>
@@ -6138,7 +6141,7 @@
       <c r="Z171" s="5"/>
       <c r="AA171" s="5"/>
     </row>
-    <row r="172" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B172" s="56">
         <v>171</v>
       </c>
@@ -6176,7 +6179,7 @@
       <c r="Z172" s="5"/>
       <c r="AA172" s="5"/>
     </row>
-    <row r="173" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B173" s="56">
         <v>172</v>
       </c>
@@ -6214,7 +6217,7 @@
       <c r="Z173" s="5"/>
       <c r="AA173" s="5"/>
     </row>
-    <row r="174" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B174" s="55">
         <v>173</v>
       </c>
@@ -6252,7 +6255,7 @@
       <c r="Z174" s="5"/>
       <c r="AA174" s="5"/>
     </row>
-    <row r="175" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B175" s="29">
         <v>174</v>
       </c>
@@ -6288,7 +6291,7 @@
       <c r="Z175" s="5"/>
       <c r="AA175" s="5"/>
     </row>
-    <row r="176" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B176" s="29">
         <v>175</v>
       </c>
@@ -6324,7 +6327,7 @@
       <c r="Z176" s="5"/>
       <c r="AA176" s="5"/>
     </row>
-    <row r="177" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B177" s="29">
         <v>176</v>
       </c>
@@ -6360,7 +6363,7 @@
       <c r="Z177" s="5"/>
       <c r="AA177" s="5"/>
     </row>
-    <row r="178" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B178" s="29">
         <v>177</v>
       </c>
@@ -6396,7 +6399,7 @@
       <c r="Z178" s="5"/>
       <c r="AA178" s="5"/>
     </row>
-    <row r="179" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B179" s="29">
         <v>178</v>
       </c>
@@ -6432,7 +6435,7 @@
       <c r="Z179" s="5"/>
       <c r="AA179" s="5"/>
     </row>
-    <row r="180" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B180" s="56">
         <v>179</v>
       </c>
@@ -6470,7 +6473,7 @@
       <c r="Z180" s="5"/>
       <c r="AA180" s="5"/>
     </row>
-    <row r="181" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B181" s="29">
         <v>180</v>
       </c>
@@ -6506,7 +6509,7 @@
       <c r="Z181" s="5"/>
       <c r="AA181" s="5"/>
     </row>
-    <row r="182" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B182" s="29">
         <v>181</v>
       </c>
@@ -6542,7 +6545,7 @@
       <c r="Z182" s="5"/>
       <c r="AA182" s="5"/>
     </row>
-    <row r="183" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B183" s="29">
         <v>182</v>
       </c>
@@ -6578,7 +6581,7 @@
       <c r="Z183" s="5"/>
       <c r="AA183" s="5"/>
     </row>
-    <row r="184" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B184" s="29">
         <v>183</v>
       </c>
@@ -6614,7 +6617,7 @@
       <c r="Z184" s="5"/>
       <c r="AA184" s="5"/>
     </row>
-    <row r="185" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B185" s="29">
         <v>184</v>
       </c>
@@ -6650,7 +6653,7 @@
       <c r="Z185" s="5"/>
       <c r="AA185" s="5"/>
     </row>
-    <row r="186" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B186" s="29">
         <v>185</v>
       </c>
@@ -6686,7 +6689,7 @@
       <c r="Z186" s="5"/>
       <c r="AA186" s="5"/>
     </row>
-    <row r="187" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B187" s="29">
         <v>186</v>
       </c>
@@ -6722,7 +6725,7 @@
       <c r="Z187" s="5"/>
       <c r="AA187" s="5"/>
     </row>
-    <row r="188" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B188" s="29">
         <v>187</v>
       </c>
@@ -6758,7 +6761,7 @@
       <c r="Z188" s="5"/>
       <c r="AA188" s="5"/>
     </row>
-    <row r="189" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B189" s="29">
         <v>188</v>
       </c>
@@ -6794,7 +6797,7 @@
       <c r="Z189" s="5"/>
       <c r="AA189" s="5"/>
     </row>
-    <row r="190" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B190" s="29">
         <v>189</v>
       </c>
@@ -6830,7 +6833,7 @@
       <c r="Z190" s="5"/>
       <c r="AA190" s="5"/>
     </row>
-    <row r="191" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B191" s="29">
         <v>190</v>
       </c>
@@ -6866,7 +6869,7 @@
       <c r="Z191" s="5"/>
       <c r="AA191" s="5"/>
     </row>
-    <row r="192" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
       <c r="B192" s="29">
         <v>191</v>
       </c>
@@ -6901,7 +6904,7 @@
       <c r="Z192" s="5"/>
       <c r="AA192" s="5"/>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B193" s="29">
         <v>192</v>
       </c>
@@ -6918,7 +6921,7 @@
       <c r="G193" s="29"/>
       <c r="H193" s="29"/>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B194" s="56">
         <v>193</v>
       </c>
@@ -6937,7 +6940,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B195" s="29">
         <v>194</v>
       </c>
@@ -6954,7 +6957,7 @@
       <c r="G195" s="29"/>
       <c r="H195" s="29"/>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B196" s="29">
         <v>195</v>
       </c>
@@ -6971,7 +6974,7 @@
       <c r="G196" s="29"/>
       <c r="H196" s="29"/>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B197" s="29">
         <v>196</v>
       </c>
@@ -6988,7 +6991,7 @@
       <c r="G197" s="29"/>
       <c r="H197" s="29"/>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B198" s="29">
         <v>197</v>
       </c>
@@ -7005,7 +7008,7 @@
       <c r="G198" s="29"/>
       <c r="H198" s="29"/>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B199" s="29">
         <v>198</v>
       </c>
@@ -7022,7 +7025,7 @@
       <c r="G199" s="29"/>
       <c r="H199" s="29"/>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B200" s="29">
         <v>199</v>
       </c>
@@ -7039,7 +7042,7 @@
       <c r="G200" s="29"/>
       <c r="H200" s="29"/>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B201" s="56">
         <v>200</v>
       </c>
@@ -7058,7 +7061,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B202" s="29">
         <v>201</v>
       </c>
@@ -7075,8 +7078,7 @@
       <c r="G202" s="29"/>
       <c r="H202" s="29"/>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A203" s="60"/>
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="B203" s="55">
         <v>202</v>
       </c>
@@ -7094,7 +7096,7 @@
       <c r="H203" s="55"/>
       <c r="I203" s="3"/>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="16"/>
       <c r="B204" s="29">
         <v>203</v>
@@ -7112,7 +7114,7 @@
       <c r="G204" s="29"/>
       <c r="H204" s="29"/>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="16"/>
       <c r="B205" s="29">
         <v>204</v>
@@ -7130,7 +7132,7 @@
       <c r="G205" s="29"/>
       <c r="H205" s="29"/>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="16"/>
       <c r="B206" s="29">
         <v>205</v>
@@ -7148,7 +7150,7 @@
       <c r="G206" s="29"/>
       <c r="H206" s="29"/>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="16"/>
       <c r="B207" s="29">
         <v>206</v>
@@ -7166,7 +7168,7 @@
       <c r="G207" s="29"/>
       <c r="H207" s="29"/>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="16"/>
       <c r="B208" s="29">
         <v>207</v>
@@ -7184,7 +7186,7 @@
       <c r="G208" s="29"/>
       <c r="H208" s="29"/>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="16"/>
       <c r="B209" s="56">
         <v>208</v>
@@ -7204,7 +7206,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="16"/>
       <c r="B210" s="29">
         <v>209</v>
@@ -7222,7 +7224,7 @@
       <c r="G210" s="29"/>
       <c r="H210" s="29"/>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="16"/>
       <c r="B211" s="29">
         <v>210</v>
@@ -7240,253 +7242,253 @@
       <c r="G211" s="29"/>
       <c r="H211" s="29"/>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B212" s="29">
         <v>211</v>
       </c>
       <c r="E212" s="20"/>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B213" s="29">
         <v>212</v>
       </c>
       <c r="E213" s="20"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B214" s="29">
         <v>213</v>
       </c>
       <c r="E214" s="22"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B215" s="29">
         <v>214</v>
       </c>
       <c r="E215" s="22"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B216" s="29">
         <v>215</v>
       </c>
       <c r="E216" s="20"/>
     </row>
-    <row r="217" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B217" s="29">
         <v>216</v>
       </c>
       <c r="E217" s="21"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B218" s="29">
         <v>217</v>
       </c>
       <c r="E218" s="20"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B219" s="29">
         <v>218</v>
       </c>
       <c r="E219" s="20"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B220" s="29">
         <v>219</v>
       </c>
       <c r="E220" s="20"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B221" s="29">
         <v>220</v>
       </c>
       <c r="E221" s="20"/>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B222" s="29">
         <v>221</v>
       </c>
       <c r="E222" s="20"/>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B223" s="29">
         <v>222</v>
       </c>
       <c r="E223" s="20"/>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
       <c r="B224" s="29">
         <v>223</v>
       </c>
       <c r="E224" s="20"/>
     </row>
-    <row r="225" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B225" s="29">
         <v>224</v>
       </c>
       <c r="E225" s="20"/>
     </row>
-    <row r="226" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B226" s="29">
         <v>225</v>
       </c>
       <c r="E226" s="20"/>
     </row>
-    <row r="227" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B227" s="29">
         <v>226</v>
       </c>
       <c r="E227" s="20"/>
     </row>
-    <row r="228" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B228" s="29">
         <v>227</v>
       </c>
       <c r="E228" s="20"/>
     </row>
-    <row r="229" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B229" s="29">
         <v>228</v>
       </c>
       <c r="E229" s="20"/>
     </row>
-    <row r="230" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B230" s="29">
         <v>229</v>
       </c>
       <c r="E230" s="20"/>
     </row>
-    <row r="231" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B231" s="29">
         <v>230</v>
       </c>
       <c r="E231" s="20"/>
     </row>
-    <row r="232" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B232" s="29">
         <v>231</v>
       </c>
       <c r="E232" s="20"/>
     </row>
-    <row r="233" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B233" s="29">
         <v>232</v>
       </c>
       <c r="E233" s="20"/>
     </row>
-    <row r="234" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B234" s="29">
         <v>233</v>
       </c>
       <c r="E234" s="20"/>
     </row>
-    <row r="235" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B235" s="29">
         <v>234</v>
       </c>
       <c r="E235" s="20"/>
     </row>
-    <row r="236" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B236" s="29">
         <v>235</v>
       </c>
       <c r="E236" s="20"/>
     </row>
-    <row r="237" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B237" s="29">
         <v>236</v>
       </c>
       <c r="E237" s="20"/>
     </row>
-    <row r="238" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B238" s="29">
         <v>237</v>
       </c>
       <c r="E238" s="20"/>
     </row>
-    <row r="239" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B239" s="29">
         <v>238</v>
       </c>
       <c r="E239" s="20"/>
     </row>
-    <row r="240" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B240" s="29">
         <v>239</v>
       </c>
       <c r="E240" s="20"/>
     </row>
-    <row r="241" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B241" s="29">
         <v>240</v>
       </c>
       <c r="E241" s="22"/>
     </row>
-    <row r="242" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B242" s="29">
         <v>241</v>
       </c>
       <c r="E242" s="22"/>
     </row>
-    <row r="243" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B243" s="29">
         <v>242</v>
       </c>
       <c r="E243" s="20"/>
     </row>
-    <row r="244" spans="2:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:5" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B244" s="29">
         <v>243</v>
       </c>
       <c r="E244" s="21"/>
     </row>
-    <row r="245" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B245" s="29">
         <v>244</v>
       </c>
       <c r="E245" s="20"/>
     </row>
-    <row r="246" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B246" s="29">
         <v>245</v>
       </c>
       <c r="E246" s="20"/>
     </row>
-    <row r="247" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B247" s="29">
         <v>246</v>
       </c>
       <c r="E247" s="20"/>
     </row>
-    <row r="248" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B248" s="29">
         <v>247</v>
       </c>
       <c r="E248" s="20"/>
     </row>
-    <row r="249" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B249" s="29">
         <v>248</v>
       </c>
       <c r="E249" s="20"/>
     </row>
-    <row r="250" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B250" s="29">
         <v>249</v>
       </c>
       <c r="E250" s="20"/>
     </row>
-    <row r="251" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B251" s="29">
         <v>250</v>
       </c>
       <c r="E251" s="20"/>
     </row>
-    <row r="252" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B252" s="29">
         <v>251</v>
       </c>
       <c r="E252" s="20"/>
     </row>
-    <row r="253" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="B253" s="29">
         <v>252</v>
       </c>
@@ -7624,7 +7626,15 @@
       <c r="D1974" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I253" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I253" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Teclado com fio"/>
+        <filter val="Teclado gamer com fio"/>
+        <filter val="Teclado sem fio"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
fix: nomes de categoria padronizados na planilha
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1638c87186bceadf/Desktop/OfertasTec/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\capta\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_AAE99CEC2896977288487518AB0B1651B879BB5B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B3FAF33-F3FF-4810-A5F4-7472D876727C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89D0BAA-3B10-4B36-BCAA-7441DE47A05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Produtos Renomear" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="511">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="511">
   <si>
     <t>Validação</t>
   </si>
@@ -626,6 +626,9 @@
     <t>https://meli.la/1ouDkYa</t>
   </si>
   <si>
+    <t>Teclado Gamer Magnético 8000hz Attack Shark Com Fio X68 He</t>
+  </si>
+  <si>
     <t>https://meli.la/2wUJ3fr</t>
   </si>
   <si>
@@ -887,7 +890,7 @@
     <t>TECHSTORE-QKZ</t>
   </si>
   <si>
-    <t>Fone gamer (headset)</t>
+    <t>Fone gamer (headset com fio)</t>
   </si>
   <si>
     <t>https://meli.la/1zm1HFa</t>
@@ -1289,7 +1292,7 @@
     <t>Pen Drive Dual Drive 2 Em 1 Usb-a E Usb-c 128gb Pendrive Tipo C Duplo Duas Entradas Gurumania</t>
   </si>
   <si>
-    <t>Mouse pad pequeno</t>
+    <t>Mousepad simples</t>
   </si>
   <si>
     <t>https://meli.la/1Z5VJQ6</t>
@@ -1554,9 +1557,6 @@
   </si>
   <si>
     <t>Vou usar os dados pra atualizar o site automaticamente.</t>
-  </si>
-  <si>
-    <t>Teclado Gamer Magnético 8000hz Attack Shark Com Fio X68 He</t>
   </si>
 </sst>
 </file>
@@ -1893,10 +1893,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2182,7 +2178,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA1974"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2226,7 +2221,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="16"/>
       <c r="B2" s="29">
         <v>1</v>
@@ -2249,7 +2244,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="16"/>
       <c r="B3" s="29">
         <v>2</v>
@@ -2272,7 +2267,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="29">
         <v>3</v>
@@ -2295,7 +2290,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="55">
         <v>4</v>
@@ -2316,7 +2311,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="16"/>
       <c r="B6" s="29">
         <v>5</v>
@@ -2339,7 +2334,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" s="29">
         <v>6</v>
@@ -2362,7 +2357,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="29">
         <v>7</v>
@@ -2385,7 +2380,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
       <c r="B9" s="29">
         <v>8</v>
@@ -2408,7 +2403,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="29">
         <v>9</v>
@@ -2431,7 +2426,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="16"/>
       <c r="B11" s="55">
         <v>10</v>
@@ -2456,7 +2451,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="16"/>
       <c r="B12" s="29">
         <v>11</v>
@@ -2479,7 +2474,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="29">
         <v>12</v>
@@ -2502,7 +2497,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="29">
         <v>13</v>
@@ -2525,7 +2520,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
       <c r="B15" s="29">
         <v>14</v>
@@ -2548,7 +2543,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="55">
         <v>15</v>
@@ -2571,7 +2566,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
       <c r="B17" s="56">
         <v>16</v>
@@ -2596,7 +2591,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="29">
         <v>17</v>
@@ -2619,7 +2614,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="16"/>
       <c r="B19" s="29">
         <v>18</v>
@@ -2642,7 +2637,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="55">
         <v>19</v>
@@ -2661,7 +2656,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="29">
         <v>20</v>
@@ -2684,7 +2679,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="55">
         <v>21</v>
@@ -2703,7 +2698,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="16"/>
       <c r="B23" s="29">
         <v>22</v>
@@ -2726,7 +2721,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="55">
         <v>23</v>
@@ -2749,7 +2744,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="55">
         <v>24</v>
@@ -2768,7 +2763,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="16"/>
       <c r="B26" s="29">
         <v>25</v>
@@ -2791,7 +2786,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="16"/>
       <c r="B27" s="29">
         <v>26</v>
@@ -2814,7 +2809,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="16"/>
       <c r="B28" s="29">
         <v>27</v>
@@ -2837,7 +2832,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="47"/>
       <c r="B29" s="48">
         <v>28</v>
@@ -2860,7 +2855,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="16"/>
       <c r="B30" s="29">
         <v>29</v>
@@ -2883,7 +2878,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="16"/>
       <c r="B31" s="29">
         <v>30</v>
@@ -2906,7 +2901,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
       <c r="B32" s="56">
         <v>31</v>
@@ -2931,7 +2926,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="55">
         <v>32</v>
@@ -2954,7 +2949,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="16"/>
       <c r="B34" s="29">
         <v>33</v>
@@ -2977,7 +2972,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="47"/>
       <c r="B35" s="48">
         <v>34</v>
@@ -3000,7 +2995,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="16"/>
       <c r="B36" s="29">
         <v>35</v>
@@ -3023,7 +3018,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="16"/>
       <c r="B37" s="29">
         <v>36</v>
@@ -3046,7 +3041,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="16"/>
       <c r="B38" s="29">
         <v>37</v>
@@ -3069,7 +3064,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="29">
         <v>38</v>
@@ -3092,7 +3087,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="16"/>
       <c r="B40" s="29">
         <v>39</v>
@@ -3115,7 +3110,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="16"/>
       <c r="B41" s="29">
         <v>40</v>
@@ -3138,7 +3133,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="55">
         <v>41</v>
@@ -3157,7 +3152,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="16"/>
       <c r="B43" s="29">
         <v>42</v>
@@ -3180,7 +3175,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="55">
         <v>43</v>
@@ -3199,7 +3194,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
       <c r="B45" s="29">
         <v>44</v>
@@ -3222,7 +3217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="29">
         <v>45</v>
@@ -3245,7 +3240,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="55">
         <v>46</v>
@@ -3268,7 +3263,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="29">
         <v>47</v>
@@ -3291,7 +3286,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="55">
         <v>48</v>
@@ -3310,7 +3305,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="29">
         <v>49</v>
@@ -3333,7 +3328,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
       <c r="B51" s="29">
         <v>50</v>
@@ -3356,7 +3351,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="29">
         <v>51</v>
@@ -3379,7 +3374,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="29">
         <v>52</v>
@@ -3402,7 +3397,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="29">
         <v>53</v>
@@ -3425,7 +3420,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="29">
         <v>54</v>
@@ -3448,7 +3443,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="29">
         <v>55</v>
@@ -4020,7 +4015,7 @@
         <v>199</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>510</v>
+        <v>200</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
@@ -4038,14 +4033,14 @@
         <v>184</v>
       </c>
       <c r="D82" s="30" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E82" s="31" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F82" s="29"/>
       <c r="G82" s="32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H82" s="29"/>
       <c r="I82" t="s">
@@ -4061,14 +4056,14 @@
         <v>184</v>
       </c>
       <c r="D83" s="34" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E83" s="35" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F83" s="33"/>
       <c r="G83" s="36" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H83" s="33" t="s">
         <v>35</v>
@@ -4086,14 +4081,14 @@
         <v>184</v>
       </c>
       <c r="D84" s="30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E84" s="31" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F84" s="29"/>
       <c r="G84" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H84" s="29"/>
       <c r="I84" t="s">
@@ -4109,14 +4104,14 @@
         <v>184</v>
       </c>
       <c r="D85" s="30" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E85" s="31" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F85" s="29"/>
       <c r="G85" s="32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H85" s="29"/>
       <c r="I85" t="s">
@@ -4132,10 +4127,10 @@
         <v>184</v>
       </c>
       <c r="D86" s="30" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E86" s="31" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F86" s="29"/>
       <c r="G86" s="32" t="s">
@@ -4155,10 +4150,10 @@
         <v>184</v>
       </c>
       <c r="D87" s="30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E87" s="31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F87" s="29"/>
       <c r="G87" s="32" t="s">
@@ -4178,122 +4173,122 @@
         <v>184</v>
       </c>
       <c r="D88" s="30" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E88" s="31" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F88" s="29"/>
       <c r="G88" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H88" s="29"/>
       <c r="I88" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="16"/>
       <c r="B89" s="29">
         <v>88</v>
       </c>
       <c r="C89" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D89" s="30" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E89" s="31" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F89" s="29"/>
       <c r="G89" s="32" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H89" s="29"/>
       <c r="I89" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="16"/>
       <c r="B90" s="29">
         <v>89</v>
       </c>
       <c r="C90" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D90" s="30" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E90" s="31" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F90" s="29"/>
       <c r="G90" s="32" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H90" s="29"/>
       <c r="I90" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="16"/>
       <c r="B91" s="29">
         <v>90</v>
       </c>
       <c r="C91" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D91" s="30" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E91" s="31" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F91" s="29"/>
       <c r="G91" s="32" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H91" s="29"/>
       <c r="I91" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="16"/>
       <c r="B92" s="29">
         <v>91</v>
       </c>
       <c r="C92" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D92" s="30" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E92" s="31" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F92" s="29"/>
       <c r="G92" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H92" s="29"/>
       <c r="I92" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="55">
         <v>92</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E93" s="6"/>
       <c r="F93" s="3"/>
@@ -4303,19 +4298,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="16"/>
       <c r="B94" s="29">
         <v>93</v>
       </c>
       <c r="C94" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D94" s="30" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E94" s="31" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F94" s="29"/>
       <c r="G94" s="32" t="s">
@@ -4326,85 +4321,85 @@
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="16"/>
       <c r="B95" s="29">
         <v>94</v>
       </c>
       <c r="C95" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D95" s="30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E95" s="31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F95" s="29"/>
       <c r="G95" s="32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H95" s="29"/>
       <c r="I95" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="16"/>
       <c r="B96" s="29">
         <v>95</v>
       </c>
       <c r="C96" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D96" s="30" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="E96" s="31" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F96" s="29"/>
       <c r="G96" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H96" s="29"/>
       <c r="I96" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="16"/>
       <c r="B97" s="29">
         <v>96</v>
       </c>
       <c r="C97" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D97" s="30" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E97" s="31" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F97" s="29"/>
       <c r="G97" s="32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H97" s="29"/>
       <c r="I97" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="55">
         <v>97</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E98" s="6"/>
       <c r="F98" s="3"/>
@@ -4414,16 +4409,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="55">
         <v>98</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E99" s="6"/>
       <c r="F99" s="3"/>
@@ -4433,131 +4428,131 @@
         <v>13</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="16"/>
       <c r="B100" s="29">
         <v>99</v>
       </c>
       <c r="C100" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D100" s="30" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E100" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F100" s="29"/>
       <c r="G100" s="32" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H100" s="29"/>
       <c r="I100" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="16"/>
       <c r="B101" s="29">
         <v>100</v>
       </c>
       <c r="C101" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D101" s="30" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E101" s="31" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F101" s="29"/>
       <c r="G101" s="32" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="H101" s="29"/>
       <c r="I101" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="16"/>
       <c r="B102" s="29">
         <v>101</v>
       </c>
       <c r="C102" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D102" s="30" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E102" s="31" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F102" s="29"/>
       <c r="G102" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H102" s="29"/>
       <c r="I102" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="55">
         <v>102</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="18" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H103" s="3"/>
       <c r="I103" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="16"/>
       <c r="B104" s="29">
         <v>103</v>
       </c>
       <c r="C104" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D104" s="30" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E104" s="31" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F104" s="29"/>
       <c r="G104" s="32" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H104" s="29"/>
       <c r="I104" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="55">
         <v>104</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E105" s="6"/>
       <c r="F105" s="3"/>
@@ -4567,85 +4562,85 @@
         <v>13</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="16"/>
       <c r="B106" s="29">
         <v>105</v>
       </c>
       <c r="C106" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D106" s="30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E106" s="31" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F106" s="29"/>
       <c r="G106" s="32" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="H106" s="29"/>
       <c r="I106" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="16"/>
       <c r="B107" s="29">
         <v>106</v>
       </c>
       <c r="C107" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D107" s="30" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E107" s="31" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F107" s="29"/>
       <c r="G107" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H107" s="29"/>
       <c r="I107" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="16"/>
       <c r="B108" s="29">
         <v>107</v>
       </c>
       <c r="C108" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D108" s="30" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E108" s="31" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F108" s="29"/>
       <c r="G108" s="32" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="H108" s="29"/>
       <c r="I108" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="55">
         <v>108</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E109" s="6"/>
       <c r="F109" s="3"/>
@@ -4655,85 +4650,85 @@
         <v>13</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="16"/>
       <c r="B110" s="29">
         <v>109</v>
       </c>
       <c r="C110" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D110" s="30" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E110" s="31" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F110" s="29"/>
       <c r="G110" s="32" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H110" s="29"/>
       <c r="I110" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="16"/>
       <c r="B111" s="29">
         <v>110</v>
       </c>
       <c r="C111" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D111" s="30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E111" s="31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F111" s="29"/>
       <c r="G111" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H111" s="29"/>
       <c r="I111" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="16"/>
       <c r="B112" s="29">
         <v>111</v>
       </c>
       <c r="C112" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D112" s="30" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E112" s="31" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F112" s="29"/>
       <c r="G112" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H112" s="29"/>
       <c r="I112" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="9"/>
       <c r="B113" s="56">
         <v>112</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E113" s="11"/>
       <c r="F113" s="9"/>
@@ -4743,108 +4738,108 @@
         <v>13</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="16"/>
       <c r="B114" s="29">
         <v>113</v>
       </c>
       <c r="C114" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D114" s="30" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E114" s="31" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F114" s="29"/>
       <c r="G114" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H114" s="29"/>
       <c r="I114" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="16"/>
       <c r="B115" s="29">
         <v>114</v>
       </c>
       <c r="C115" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D115" s="30" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E115" s="31" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F115" s="29"/>
       <c r="G115" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H115" s="29"/>
       <c r="I115" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="16"/>
       <c r="B116" s="29">
         <v>115</v>
       </c>
       <c r="C116" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D116" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E116" s="31" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F116" s="29"/>
       <c r="G116" s="29" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="H116" s="29"/>
       <c r="I116" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="16"/>
       <c r="B117" s="29">
         <v>116</v>
       </c>
       <c r="C117" s="29" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D117" s="30" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E117" s="31" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F117" s="29"/>
       <c r="G117" s="32" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="H117" s="29"/>
       <c r="I117" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="3"/>
       <c r="B118" s="55">
         <v>117</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E118" s="6"/>
       <c r="F118" s="3"/>
@@ -4854,19 +4849,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="16"/>
       <c r="B119" s="29">
         <v>118</v>
       </c>
       <c r="C119" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D119" s="30" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E119" s="31" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F119" s="29"/>
       <c r="G119" s="32" t="s">
@@ -4877,19 +4872,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="16"/>
       <c r="B120" s="29">
         <v>119</v>
       </c>
       <c r="C120" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D120" s="30" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E120" s="31" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F120" s="29"/>
       <c r="G120" s="32" t="s">
@@ -4900,19 +4895,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="16"/>
       <c r="B121" s="29">
         <v>120</v>
       </c>
       <c r="C121" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D121" s="30" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E121" s="31" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F121" s="29"/>
       <c r="G121" s="32" t="s">
@@ -4923,16 +4918,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="3"/>
       <c r="B122" s="55">
         <v>121</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E122" s="6"/>
       <c r="F122" s="3"/>
@@ -4942,88 +4937,88 @@
         <v>13</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="16"/>
       <c r="B123" s="29">
         <v>122</v>
       </c>
       <c r="C123" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D123" s="30" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E123" s="31" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F123" s="29"/>
       <c r="G123" s="32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H123" s="29"/>
       <c r="I123" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="16"/>
       <c r="B124" s="29">
         <v>123</v>
       </c>
       <c r="C124" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D124" s="30" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E124" s="31" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F124" s="29"/>
       <c r="G124" s="29" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H124" s="29"/>
       <c r="I124" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="12"/>
       <c r="B125" s="29">
         <v>124</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E125" s="14" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F125" s="12"/>
       <c r="G125" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H125" s="12"/>
       <c r="I125" s="12" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="16"/>
       <c r="B126" s="29">
         <v>125</v>
       </c>
       <c r="C126" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D126" s="30" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E126" s="31" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F126" s="29"/>
       <c r="G126" s="29" t="s">
@@ -5034,19 +5029,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="16"/>
       <c r="B127" s="29">
         <v>126</v>
       </c>
       <c r="C127" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D127" s="30" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E127" s="31" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F127" s="29"/>
       <c r="G127" s="32" t="s">
@@ -5057,19 +5052,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="16"/>
       <c r="B128" s="29">
         <v>127</v>
       </c>
       <c r="C128" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D128" s="30" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E128" s="31" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F128" s="29"/>
       <c r="G128" s="29" t="s">
@@ -5080,42 +5075,42 @@
         <v>13</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="16"/>
       <c r="B129" s="29">
         <v>128</v>
       </c>
       <c r="C129" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D129" s="30" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E129" s="31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F129" s="29"/>
       <c r="G129" s="32" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="H129" s="29"/>
       <c r="I129" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="16"/>
       <c r="B130" s="29">
         <v>129</v>
       </c>
       <c r="C130" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D130" s="30" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E130" s="29" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F130" s="29"/>
       <c r="G130" s="32" t="s">
@@ -5126,19 +5121,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="16"/>
       <c r="B131" s="29">
         <v>130</v>
       </c>
       <c r="C131" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D131" s="30" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E131" s="29" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F131" s="29"/>
       <c r="G131" s="32" t="s">
@@ -5149,19 +5144,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="16"/>
       <c r="B132" s="29">
         <v>131</v>
       </c>
       <c r="C132" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D132" s="30" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E132" s="31" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F132" s="29"/>
       <c r="G132" s="32" t="s">
@@ -5172,265 +5167,263 @@
         <v>13</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="16"/>
       <c r="B133" s="29">
         <v>132</v>
       </c>
       <c r="C133" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D133" s="30" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E133" s="31" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F133" s="29"/>
       <c r="G133" s="32" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H133" s="29"/>
       <c r="I133" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="16"/>
       <c r="B134" s="29">
         <v>133</v>
       </c>
       <c r="C134" s="29" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D134" s="30" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E134" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F134" s="29"/>
       <c r="G134" s="32" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H134" s="29"/>
       <c r="I134" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="16"/>
       <c r="B135" s="29">
         <v>134</v>
       </c>
       <c r="C135" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D135" s="30" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E135" s="31" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F135" s="29"/>
       <c r="G135" s="32" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H135" s="29"/>
       <c r="I135" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="16"/>
       <c r="B136" s="29">
         <v>135</v>
       </c>
       <c r="C136" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D136" s="30" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E136" s="31" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F136" s="29"/>
       <c r="G136" s="32" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H136" s="29"/>
       <c r="I136" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="16"/>
       <c r="B137" s="29">
         <v>136</v>
       </c>
       <c r="C137" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D137" s="30" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E137" s="31" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F137" s="29"/>
       <c r="G137" s="32" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H137" s="29"/>
       <c r="I137" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="16"/>
-      <c r="B138" s="33">
+      <c r="B138" s="29">
         <v>137</v>
       </c>
-      <c r="C138" s="33" t="s">
-        <v>325</v>
-      </c>
-      <c r="D138" s="34" t="s">
-        <v>334</v>
-      </c>
-      <c r="E138" s="35" t="s">
+      <c r="C138" s="29" t="s">
+        <v>326</v>
+      </c>
+      <c r="D138" s="30" t="s">
         <v>335</v>
       </c>
-      <c r="F138" s="33"/>
-      <c r="G138" s="36" t="s">
-        <v>221</v>
-      </c>
-      <c r="H138" s="33" t="s">
-        <v>35</v>
-      </c>
+      <c r="E138" s="31" t="s">
+        <v>336</v>
+      </c>
+      <c r="F138" s="29"/>
+      <c r="G138" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="H138" s="29"/>
       <c r="I138" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="16"/>
       <c r="B139" s="29">
         <v>138</v>
       </c>
       <c r="C139" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D139" s="30" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E139" s="31" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F139" s="29"/>
       <c r="G139" s="32" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H139" s="29"/>
       <c r="I139" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="16"/>
       <c r="B140" s="29">
         <v>139</v>
       </c>
       <c r="C140" s="29" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D140" s="30" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="E140" s="31" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F140" s="29"/>
       <c r="G140" s="32" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H140" s="29"/>
       <c r="I140" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="141" spans="1:9" s="57" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" s="57" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="16"/>
       <c r="B141" s="29">
         <v>140</v>
       </c>
       <c r="C141" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D141" s="41" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E141" s="31" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F141" s="29"/>
       <c r="G141" s="32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="H141" s="29"/>
     </row>
-    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="16"/>
       <c r="B142" s="29">
         <v>141</v>
       </c>
       <c r="C142" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D142" s="41" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E142" s="31" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F142" s="29"/>
       <c r="G142" s="32" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H142" s="29"/>
     </row>
-    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="16"/>
       <c r="B143" s="29">
         <v>142</v>
       </c>
       <c r="C143" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D143" s="41" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E143" s="31" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F143" s="29"/>
       <c r="G143" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H143" s="29"/>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="16"/>
       <c r="B144" s="29">
         <v>143</v>
       </c>
       <c r="C144" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D144" s="41" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E144" s="31" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F144" s="29"/>
       <c r="G144" s="32" t="s">
@@ -5438,101 +5431,101 @@
       </c>
       <c r="H144" s="29"/>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="9"/>
       <c r="B145" s="56">
         <v>144</v>
       </c>
       <c r="C145" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D145" s="43" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E145" s="39" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F145" s="37"/>
       <c r="G145" s="40" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H145" s="37" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="16"/>
       <c r="B146" s="29">
         <v>145</v>
       </c>
       <c r="C146" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D146" s="41" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E146" s="31" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F146" s="29"/>
       <c r="G146" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H146" s="29"/>
     </row>
-    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="16"/>
       <c r="B147" s="29">
         <v>146</v>
       </c>
       <c r="C147" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D147" s="41" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E147" s="31" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F147" s="29"/>
       <c r="G147" s="32" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="H147" s="29"/>
     </row>
-    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="16"/>
       <c r="B148" s="29">
         <v>147</v>
       </c>
       <c r="C148" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D148" s="41" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E148" s="31" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F148" s="29"/>
       <c r="G148" s="32" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H148" s="29"/>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="16"/>
       <c r="B149" s="29">
         <v>148</v>
       </c>
       <c r="C149" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D149" s="41" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E149" s="31" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F149" s="29"/>
       <c r="G149" s="32" t="s">
@@ -5540,195 +5533,195 @@
       </c>
       <c r="H149" s="29"/>
     </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="9"/>
       <c r="B150" s="56">
         <v>149</v>
       </c>
       <c r="C150" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D150" s="43" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E150" s="39" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F150" s="37"/>
       <c r="G150" s="40" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H150" s="37" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="151" spans="1:9" s="47" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" s="47" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B151" s="48">
         <v>150</v>
       </c>
       <c r="C151" s="48" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D151" s="54" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E151" s="50" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F151" s="48"/>
       <c r="G151" s="51" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="H151" s="48"/>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="16"/>
       <c r="B152" s="29">
         <v>151</v>
       </c>
       <c r="C152" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D152" s="41" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E152" s="31" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F152" s="31"/>
       <c r="G152" s="32" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="H152" s="29"/>
     </row>
-    <row r="153" spans="1:9" ht="21.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A153" s="16"/>
       <c r="B153" s="29">
         <v>152</v>
       </c>
       <c r="C153" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D153" s="41" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E153" s="31" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F153" s="44"/>
       <c r="G153" s="32" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H153" s="29"/>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="16"/>
       <c r="B154" s="29">
         <v>153</v>
       </c>
       <c r="C154" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D154" s="41" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E154" s="31" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F154" s="31"/>
       <c r="G154" s="32" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H154" s="29"/>
     </row>
-    <row r="155" spans="1:9" ht="21.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="9"/>
       <c r="B155" s="56">
         <v>154</v>
       </c>
       <c r="C155" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D155" s="43" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E155" s="39" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F155" s="45"/>
       <c r="G155" s="40" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H155" s="37" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="3"/>
       <c r="B156" s="55">
         <v>155</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F156" s="6"/>
       <c r="G156" s="3"/>
       <c r="H156" s="3"/>
       <c r="I156" s="3"/>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="16"/>
       <c r="B157" s="29">
         <v>156</v>
       </c>
       <c r="C157" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D157" s="41" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E157" s="31" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F157" s="29"/>
       <c r="G157" s="29"/>
       <c r="H157" s="29"/>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B158" s="29">
         <v>157</v>
       </c>
       <c r="C158" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D158" s="41" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E158" s="31" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F158" s="29"/>
       <c r="G158" s="29"/>
       <c r="H158" s="29"/>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B159" s="56">
         <v>158</v>
       </c>
       <c r="C159" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D159" s="43" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E159" s="39" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F159" s="37"/>
       <c r="G159" s="37"/>
@@ -5736,18 +5729,18 @@
         <v>53</v>
       </c>
     </row>
-    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B160" s="56">
         <v>159</v>
       </c>
       <c r="C160" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D160" s="43" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E160" s="39" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F160" s="37"/>
       <c r="G160" s="37"/>
@@ -5755,36 +5748,36 @@
         <v>53</v>
       </c>
     </row>
-    <row r="161" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B161" s="29">
         <v>160</v>
       </c>
       <c r="C161" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D161" s="41" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E161" s="31" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F161" s="31"/>
       <c r="G161" s="31"/>
       <c r="H161" s="31"/>
       <c r="I161" s="5"/>
     </row>
-    <row r="162" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B162" s="56">
         <v>161</v>
       </c>
       <c r="C162" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D162" s="43" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E162" s="39" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F162" s="39"/>
       <c r="G162" s="39"/>
@@ -5811,19 +5804,19 @@
       <c r="Z162" s="5"/>
       <c r="AA162" s="5"/>
     </row>
-    <row r="163" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
       <c r="B163" s="55">
         <v>162</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D163" s="25" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F163" s="6"/>
       <c r="G163" s="6"/>
@@ -5848,19 +5841,19 @@
       <c r="Z163" s="5"/>
       <c r="AA163" s="5"/>
     </row>
-    <row r="164" spans="1:27" s="3" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:27" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="26"/>
       <c r="B164" s="56">
         <v>163</v>
       </c>
       <c r="C164" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D164" s="43" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E164" s="39" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F164" s="39"/>
       <c r="G164" s="39"/>
@@ -5887,18 +5880,18 @@
       <c r="Z164" s="5"/>
       <c r="AA164" s="5"/>
     </row>
-    <row r="165" spans="1:27" s="26" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:27" s="26" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B165" s="29">
         <v>164</v>
       </c>
       <c r="C165" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D165" s="41" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E165" s="31" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F165" s="31"/>
       <c r="G165" s="31"/>
@@ -5923,18 +5916,18 @@
       <c r="Z165" s="5"/>
       <c r="AA165" s="5"/>
     </row>
-    <row r="166" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B166" s="29">
         <v>165</v>
       </c>
       <c r="C166" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D166" s="41" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E166" s="31" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F166" s="31"/>
       <c r="G166" s="31"/>
@@ -5959,18 +5952,18 @@
       <c r="Z166" s="5"/>
       <c r="AA166" s="5"/>
     </row>
-    <row r="167" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B167" s="29">
         <v>166</v>
       </c>
       <c r="C167" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D167" s="41" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E167" s="31" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F167" s="31"/>
       <c r="G167" s="31"/>
@@ -5995,18 +5988,18 @@
       <c r="Z167" s="5"/>
       <c r="AA167" s="5"/>
     </row>
-    <row r="168" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B168" s="29">
         <v>167</v>
       </c>
       <c r="C168" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D168" s="41" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E168" s="31" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F168" s="31"/>
       <c r="G168" s="31"/>
@@ -6031,18 +6024,18 @@
       <c r="Z168" s="5"/>
       <c r="AA168" s="5"/>
     </row>
-    <row r="169" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B169" s="56">
         <v>168</v>
       </c>
       <c r="C169" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D169" s="43" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E169" s="39" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F169" s="39"/>
       <c r="G169" s="39"/>
@@ -6069,18 +6062,18 @@
       <c r="Z169" s="5"/>
       <c r="AA169" s="5"/>
     </row>
-    <row r="170" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B170" s="29">
         <v>169</v>
       </c>
       <c r="C170" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D170" s="41" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E170" s="31" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F170" s="31"/>
       <c r="G170" s="31"/>
@@ -6105,18 +6098,18 @@
       <c r="Z170" s="5"/>
       <c r="AA170" s="5"/>
     </row>
-    <row r="171" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B171" s="29">
         <v>170</v>
       </c>
       <c r="C171" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D171" s="41" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E171" s="31" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F171" s="31"/>
       <c r="G171" s="31"/>
@@ -6141,18 +6134,18 @@
       <c r="Z171" s="5"/>
       <c r="AA171" s="5"/>
     </row>
-    <row r="172" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B172" s="56">
         <v>171</v>
       </c>
       <c r="C172" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D172" s="43" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E172" s="39" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F172" s="39"/>
       <c r="G172" s="39"/>
@@ -6179,18 +6172,18 @@
       <c r="Z172" s="5"/>
       <c r="AA172" s="5"/>
     </row>
-    <row r="173" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B173" s="56">
         <v>172</v>
       </c>
       <c r="C173" s="37" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D173" s="43" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E173" s="39" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F173" s="39"/>
       <c r="G173" s="39"/>
@@ -6217,18 +6210,18 @@
       <c r="Z173" s="5"/>
       <c r="AA173" s="5"/>
     </row>
-    <row r="174" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B174" s="55">
         <v>173</v>
       </c>
       <c r="C174" s="33" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D174" s="46" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E174" s="35" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F174" s="35"/>
       <c r="G174" s="35"/>
@@ -6255,18 +6248,18 @@
       <c r="Z174" s="5"/>
       <c r="AA174" s="5"/>
     </row>
-    <row r="175" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B175" s="29">
         <v>174</v>
       </c>
       <c r="C175" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D175" s="41" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E175" s="31" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F175" s="31"/>
       <c r="G175" s="31"/>
@@ -6291,18 +6284,18 @@
       <c r="Z175" s="5"/>
       <c r="AA175" s="5"/>
     </row>
-    <row r="176" spans="1:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B176" s="29">
         <v>175</v>
       </c>
       <c r="C176" s="29" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D176" s="41" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E176" s="31" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="F176" s="31"/>
       <c r="G176" s="31"/>
@@ -6327,18 +6320,18 @@
       <c r="Z176" s="5"/>
       <c r="AA176" s="5"/>
     </row>
-    <row r="177" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B177" s="29">
         <v>176</v>
       </c>
       <c r="C177" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D177" s="41" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E177" s="31" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F177" s="31"/>
       <c r="G177" s="31"/>
@@ -6363,18 +6356,18 @@
       <c r="Z177" s="5"/>
       <c r="AA177" s="5"/>
     </row>
-    <row r="178" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B178" s="29">
         <v>177</v>
       </c>
       <c r="C178" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D178" s="41" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E178" s="31" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F178" s="31"/>
       <c r="G178" s="31"/>
@@ -6399,18 +6392,18 @@
       <c r="Z178" s="5"/>
       <c r="AA178" s="5"/>
     </row>
-    <row r="179" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B179" s="29">
         <v>178</v>
       </c>
       <c r="C179" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D179" s="41" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E179" s="31" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F179" s="31"/>
       <c r="G179" s="31"/>
@@ -6435,18 +6428,18 @@
       <c r="Z179" s="5"/>
       <c r="AA179" s="5"/>
     </row>
-    <row r="180" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B180" s="56">
         <v>179</v>
       </c>
       <c r="C180" s="37" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D180" s="43" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E180" s="39" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F180" s="39"/>
       <c r="G180" s="39"/>
@@ -6473,18 +6466,18 @@
       <c r="Z180" s="5"/>
       <c r="AA180" s="5"/>
     </row>
-    <row r="181" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B181" s="29">
         <v>180</v>
       </c>
       <c r="C181" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D181" s="41" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E181" s="31" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F181" s="31"/>
       <c r="G181" s="31"/>
@@ -6509,18 +6502,18 @@
       <c r="Z181" s="5"/>
       <c r="AA181" s="5"/>
     </row>
-    <row r="182" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B182" s="29">
         <v>181</v>
       </c>
       <c r="C182" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D182" s="41" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E182" s="31" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F182" s="31"/>
       <c r="G182" s="31"/>
@@ -6545,18 +6538,18 @@
       <c r="Z182" s="5"/>
       <c r="AA182" s="5"/>
     </row>
-    <row r="183" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B183" s="29">
         <v>182</v>
       </c>
       <c r="C183" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D183" s="41" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E183" s="31" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F183" s="31"/>
       <c r="G183" s="31"/>
@@ -6581,18 +6574,18 @@
       <c r="Z183" s="5"/>
       <c r="AA183" s="5"/>
     </row>
-    <row r="184" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B184" s="29">
         <v>183</v>
       </c>
       <c r="C184" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D184" s="41" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E184" s="31" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F184" s="31"/>
       <c r="G184" s="31"/>
@@ -6617,18 +6610,18 @@
       <c r="Z184" s="5"/>
       <c r="AA184" s="5"/>
     </row>
-    <row r="185" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B185" s="29">
         <v>184</v>
       </c>
       <c r="C185" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D185" s="41" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E185" s="31" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F185" s="31"/>
       <c r="G185" s="31"/>
@@ -6653,18 +6646,18 @@
       <c r="Z185" s="5"/>
       <c r="AA185" s="5"/>
     </row>
-    <row r="186" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B186" s="29">
         <v>185</v>
       </c>
       <c r="C186" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D186" s="41" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="E186" s="31" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F186" s="31"/>
       <c r="G186" s="31"/>
@@ -6689,18 +6682,18 @@
       <c r="Z186" s="5"/>
       <c r="AA186" s="5"/>
     </row>
-    <row r="187" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B187" s="29">
         <v>186</v>
       </c>
       <c r="C187" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D187" s="41" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E187" s="31" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F187" s="31"/>
       <c r="G187" s="31"/>
@@ -6725,18 +6718,18 @@
       <c r="Z187" s="5"/>
       <c r="AA187" s="5"/>
     </row>
-    <row r="188" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B188" s="29">
         <v>187</v>
       </c>
       <c r="C188" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D188" s="41" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E188" s="31" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="F188" s="31"/>
       <c r="G188" s="31"/>
@@ -6761,18 +6754,18 @@
       <c r="Z188" s="5"/>
       <c r="AA188" s="5"/>
     </row>
-    <row r="189" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B189" s="29">
         <v>188</v>
       </c>
       <c r="C189" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D189" s="41" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E189" s="31" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F189" s="31"/>
       <c r="G189" s="31"/>
@@ -6797,18 +6790,18 @@
       <c r="Z189" s="5"/>
       <c r="AA189" s="5"/>
     </row>
-    <row r="190" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B190" s="29">
         <v>189</v>
       </c>
       <c r="C190" s="29" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D190" s="41" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E190" s="31" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F190" s="31"/>
       <c r="G190" s="31"/>
@@ -6833,18 +6826,18 @@
       <c r="Z190" s="5"/>
       <c r="AA190" s="5"/>
     </row>
-    <row r="191" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B191" s="29">
         <v>190</v>
       </c>
       <c r="C191" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D191" s="41" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E191" s="31" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F191" s="31"/>
       <c r="G191" s="31"/>
@@ -6869,18 +6862,18 @@
       <c r="Z191" s="5"/>
       <c r="AA191" s="5"/>
     </row>
-    <row r="192" spans="2:27" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B192" s="29">
         <v>191</v>
       </c>
       <c r="C192" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D192" s="41" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E192" s="31" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F192" s="29"/>
       <c r="G192" s="29"/>
@@ -6904,35 +6897,35 @@
       <c r="Z192" s="5"/>
       <c r="AA192" s="5"/>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B193" s="29">
         <v>192</v>
       </c>
       <c r="C193" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D193" s="41" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E193" s="31" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F193" s="29"/>
       <c r="G193" s="29"/>
       <c r="H193" s="29"/>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B194" s="56">
         <v>193</v>
       </c>
       <c r="C194" s="37" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D194" s="43" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E194" s="39" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F194" s="37"/>
       <c r="G194" s="37"/>
@@ -6940,120 +6933,120 @@
         <v>53</v>
       </c>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B195" s="29">
         <v>194</v>
       </c>
       <c r="C195" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D195" s="41" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E195" s="31" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F195" s="29"/>
       <c r="G195" s="29"/>
       <c r="H195" s="29"/>
     </row>
-    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B196" s="29">
         <v>195</v>
       </c>
       <c r="C196" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D196" s="41" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="E196" s="31" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F196" s="29"/>
       <c r="G196" s="29"/>
       <c r="H196" s="29"/>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B197" s="29">
         <v>196</v>
       </c>
       <c r="C197" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D197" s="41" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E197" s="31" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F197" s="29"/>
       <c r="G197" s="29"/>
       <c r="H197" s="29"/>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B198" s="29">
         <v>197</v>
       </c>
       <c r="C198" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D198" s="41" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E198" s="31" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F198" s="29"/>
       <c r="G198" s="29"/>
       <c r="H198" s="29"/>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B199" s="29">
         <v>198</v>
       </c>
       <c r="C199" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D199" s="41" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E199" s="31" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F199" s="29"/>
       <c r="G199" s="29"/>
       <c r="H199" s="29"/>
     </row>
-    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B200" s="29">
         <v>199</v>
       </c>
       <c r="C200" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D200" s="41" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E200" s="31" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F200" s="29"/>
       <c r="G200" s="29"/>
       <c r="H200" s="29"/>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B201" s="56">
         <v>200</v>
       </c>
       <c r="C201" s="37" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D201" s="43" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E201" s="39" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F201" s="37"/>
       <c r="G201" s="37"/>
@@ -7061,24 +7054,24 @@
         <v>53</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B202" s="29">
         <v>201</v>
       </c>
       <c r="C202" s="29" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D202" s="41" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E202" s="31" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F202" s="29"/>
       <c r="G202" s="29"/>
       <c r="H202" s="29"/>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B203" s="55">
         <v>202</v>
       </c>
@@ -7086,17 +7079,17 @@
         <v>9</v>
       </c>
       <c r="D203" s="58" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E203" s="59" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F203" s="55"/>
       <c r="G203" s="55"/>
       <c r="H203" s="55"/>
       <c r="I203" s="3"/>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" s="16"/>
       <c r="B204" s="29">
         <v>203</v>
@@ -7105,16 +7098,16 @@
         <v>9</v>
       </c>
       <c r="D204" s="41" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E204" s="31" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F204" s="29"/>
       <c r="G204" s="29"/>
       <c r="H204" s="29"/>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" s="16"/>
       <c r="B205" s="29">
         <v>204</v>
@@ -7123,16 +7116,16 @@
         <v>9</v>
       </c>
       <c r="D205" s="41" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E205" s="31" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F205" s="29"/>
       <c r="G205" s="29"/>
       <c r="H205" s="29"/>
     </row>
-    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" s="16"/>
       <c r="B206" s="29">
         <v>205</v>
@@ -7141,16 +7134,16 @@
         <v>9</v>
       </c>
       <c r="D206" s="41" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E206" s="31" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F206" s="29"/>
       <c r="G206" s="29"/>
       <c r="H206" s="29"/>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" s="16"/>
       <c r="B207" s="29">
         <v>206</v>
@@ -7159,16 +7152,16 @@
         <v>9</v>
       </c>
       <c r="D207" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E207" s="31" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F207" s="29"/>
       <c r="G207" s="29"/>
       <c r="H207" s="29"/>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" s="16"/>
       <c r="B208" s="29">
         <v>207</v>
@@ -7177,16 +7170,16 @@
         <v>9</v>
       </c>
       <c r="D208" s="41" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E208" s="31" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F208" s="29"/>
       <c r="G208" s="29"/>
       <c r="H208" s="29"/>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="16"/>
       <c r="B209" s="56">
         <v>208</v>
@@ -7195,10 +7188,10 @@
         <v>9</v>
       </c>
       <c r="D209" s="43" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E209" s="39" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F209" s="37"/>
       <c r="G209" s="37"/>
@@ -7206,7 +7199,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="16"/>
       <c r="B210" s="29">
         <v>209</v>
@@ -7215,16 +7208,16 @@
         <v>9</v>
       </c>
       <c r="D210" s="41" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E210" s="31" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F210" s="29"/>
       <c r="G210" s="29"/>
       <c r="H210" s="29"/>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="16"/>
       <c r="B211" s="29">
         <v>210</v>
@@ -7233,262 +7226,262 @@
         <v>9</v>
       </c>
       <c r="D211" s="41" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E211" s="31" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F211" s="29"/>
       <c r="G211" s="29"/>
       <c r="H211" s="29"/>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B212" s="29">
         <v>211</v>
       </c>
       <c r="E212" s="20"/>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B213" s="29">
         <v>212</v>
       </c>
       <c r="E213" s="20"/>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B214" s="29">
         <v>213</v>
       </c>
       <c r="E214" s="22"/>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B215" s="29">
         <v>214</v>
       </c>
       <c r="E215" s="22"/>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B216" s="29">
         <v>215</v>
       </c>
       <c r="E216" s="20"/>
     </row>
-    <row r="217" spans="1:8" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B217" s="29">
         <v>216</v>
       </c>
       <c r="E217" s="21"/>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B218" s="29">
         <v>217</v>
       </c>
       <c r="E218" s="20"/>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B219" s="29">
         <v>218</v>
       </c>
       <c r="E219" s="20"/>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B220" s="29">
         <v>219</v>
       </c>
       <c r="E220" s="20"/>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B221" s="29">
         <v>220</v>
       </c>
       <c r="E221" s="20"/>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B222" s="29">
         <v>221</v>
       </c>
       <c r="E222" s="20"/>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B223" s="29">
         <v>222</v>
       </c>
       <c r="E223" s="20"/>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B224" s="29">
         <v>223</v>
       </c>
       <c r="E224" s="20"/>
     </row>
-    <row r="225" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B225" s="29">
         <v>224</v>
       </c>
       <c r="E225" s="20"/>
     </row>
-    <row r="226" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B226" s="29">
         <v>225</v>
       </c>
       <c r="E226" s="20"/>
     </row>
-    <row r="227" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B227" s="29">
         <v>226</v>
       </c>
       <c r="E227" s="20"/>
     </row>
-    <row r="228" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B228" s="29">
         <v>227</v>
       </c>
       <c r="E228" s="20"/>
     </row>
-    <row r="229" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B229" s="29">
         <v>228</v>
       </c>
       <c r="E229" s="20"/>
     </row>
-    <row r="230" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B230" s="29">
         <v>229</v>
       </c>
       <c r="E230" s="20"/>
     </row>
-    <row r="231" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B231" s="29">
         <v>230</v>
       </c>
       <c r="E231" s="20"/>
     </row>
-    <row r="232" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B232" s="29">
         <v>231</v>
       </c>
       <c r="E232" s="20"/>
     </row>
-    <row r="233" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B233" s="29">
         <v>232</v>
       </c>
       <c r="E233" s="20"/>
     </row>
-    <row r="234" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B234" s="29">
         <v>233</v>
       </c>
       <c r="E234" s="20"/>
     </row>
-    <row r="235" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B235" s="29">
         <v>234</v>
       </c>
       <c r="E235" s="20"/>
     </row>
-    <row r="236" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B236" s="29">
         <v>235</v>
       </c>
       <c r="E236" s="20"/>
     </row>
-    <row r="237" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B237" s="29">
         <v>236</v>
       </c>
       <c r="E237" s="20"/>
     </row>
-    <row r="238" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B238" s="29">
         <v>237</v>
       </c>
       <c r="E238" s="20"/>
     </row>
-    <row r="239" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B239" s="29">
         <v>238</v>
       </c>
       <c r="E239" s="20"/>
     </row>
-    <row r="240" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B240" s="29">
         <v>239</v>
       </c>
       <c r="E240" s="20"/>
     </row>
-    <row r="241" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B241" s="29">
         <v>240</v>
       </c>
       <c r="E241" s="22"/>
     </row>
-    <row r="242" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B242" s="29">
         <v>241</v>
       </c>
       <c r="E242" s="22"/>
     </row>
-    <row r="243" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B243" s="29">
         <v>242</v>
       </c>
       <c r="E243" s="20"/>
     </row>
-    <row r="244" spans="2:5" ht="15.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B244" s="29">
         <v>243</v>
       </c>
       <c r="E244" s="21"/>
     </row>
-    <row r="245" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B245" s="29">
         <v>244</v>
       </c>
       <c r="E245" s="20"/>
     </row>
-    <row r="246" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B246" s="29">
         <v>245</v>
       </c>
       <c r="E246" s="20"/>
     </row>
-    <row r="247" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B247" s="29">
         <v>246</v>
       </c>
       <c r="E247" s="20"/>
     </row>
-    <row r="248" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B248" s="29">
         <v>247</v>
       </c>
       <c r="E248" s="20"/>
     </row>
-    <row r="249" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B249" s="29">
         <v>248</v>
       </c>
       <c r="E249" s="20"/>
     </row>
-    <row r="250" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B250" s="29">
         <v>249</v>
       </c>
       <c r="E250" s="20"/>
     </row>
-    <row r="251" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B251" s="29">
         <v>250</v>
       </c>
       <c r="E251" s="20"/>
     </row>
-    <row r="252" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B252" s="29">
         <v>251</v>
       </c>
       <c r="E252" s="20"/>
     </row>
-    <row r="253" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B253" s="29">
         <v>252</v>
       </c>
@@ -7626,15 +7619,6 @@
       <c r="D1974" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I253" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Teclado com fio"/>
-        <filter val="Teclado gamer com fio"/>
-        <filter val="Teclado sem fio"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -7861,92 +7845,92 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adicionando os mouses gamer sem fio corretamente
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -1387,31 +1387,31 @@
     </row>
     <row r="21">
       <c r="A21" s="16" t="n"/>
-      <c r="B21" s="36" t="n">
+      <c r="B21" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="C21" s="36" t="inlineStr">
+      <c r="C21" s="28" t="inlineStr">
         <is>
           <t>Mouse gamer sem fio</t>
         </is>
       </c>
-      <c r="D21" s="42" t="inlineStr">
+      <c r="D21" s="40" t="inlineStr">
         <is>
           <t>https://meli.la/2eiaX1o</t>
         </is>
       </c>
-      <c r="E21" s="38" t="inlineStr">
+      <c r="E21" s="30" t="inlineStr">
         <is>
           <t>Mouse Gamer Attack Shark R1 Sem Fio</t>
         </is>
       </c>
-      <c r="F21" s="36" t="n"/>
-      <c r="G21" s="36" t="inlineStr">
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="inlineStr">
         <is>
           <t>Attack Shark</t>
         </is>
       </c>
-      <c r="H21" s="36" t="inlineStr">
+      <c r="H21" s="28" t="inlineStr">
         <is>
           <t>estoque baixo</t>
         </is>
@@ -1453,31 +1453,35 @@
     </row>
     <row r="23">
       <c r="A23" s="16" t="n"/>
-      <c r="B23" s="28" t="n">
+      <c r="B23" s="36" t="n">
         <v>22</v>
       </c>
-      <c r="C23" s="28" t="inlineStr">
+      <c r="C23" s="36" t="inlineStr">
         <is>
           <t>Mouse gamer sem fio</t>
         </is>
       </c>
-      <c r="D23" s="29" t="inlineStr">
+      <c r="D23" s="37" t="inlineStr">
         <is>
           <t>https://meli.la/1ViXRN7</t>
         </is>
       </c>
-      <c r="E23" s="30" t="inlineStr">
+      <c r="E23" s="38" t="inlineStr">
         <is>
           <t>Mouse Gamer Attack Shark R1 Branco</t>
         </is>
       </c>
-      <c r="F23" s="28" t="n"/>
-      <c r="G23" s="28" t="inlineStr">
+      <c r="F23" s="36" t="n"/>
+      <c r="G23" s="36" t="inlineStr">
         <is>
           <t>Attack Shark</t>
         </is>
       </c>
-      <c r="H23" s="28" t="n"/>
+      <c r="H23" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>⬜</t>
@@ -1581,31 +1585,35 @@
     </row>
     <row r="27">
       <c r="A27" s="16" t="n"/>
-      <c r="B27" s="28" t="n">
+      <c r="B27" s="36" t="n">
         <v>26</v>
       </c>
-      <c r="C27" s="28" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>Mouse gamer sem fio</t>
         </is>
       </c>
-      <c r="D27" s="29" t="inlineStr">
+      <c r="D27" s="37" t="inlineStr">
         <is>
           <t>https://meli.la/2iuRXex</t>
         </is>
       </c>
-      <c r="E27" s="30" t="inlineStr">
+      <c r="E27" s="38" t="inlineStr">
         <is>
           <t>Mouse Gamer Redragon King Pro 4K</t>
         </is>
       </c>
-      <c r="F27" s="28" t="n"/>
-      <c r="G27" s="28" t="inlineStr">
+      <c r="F27" s="36" t="n"/>
+      <c r="G27" s="36" t="inlineStr">
         <is>
           <t>Redragon</t>
         </is>
       </c>
-      <c r="H27" s="28" t="n"/>
+      <c r="H27" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>⬜</t>
@@ -1684,31 +1692,31 @@
     </row>
     <row r="30">
       <c r="A30" s="16" t="n"/>
-      <c r="B30" s="36" t="n">
+      <c r="B30" s="28" t="n">
         <v>29</v>
       </c>
-      <c r="C30" s="36" t="inlineStr">
+      <c r="C30" s="28" t="inlineStr">
         <is>
           <t>Mouse gamer sem fio</t>
         </is>
       </c>
-      <c r="D30" s="37" t="inlineStr">
+      <c r="D30" s="29" t="inlineStr">
         <is>
           <t>https://meli.la/2kvFciT</t>
         </is>
       </c>
-      <c r="E30" s="38" t="inlineStr">
+      <c r="E30" s="30" t="inlineStr">
         <is>
           <t>Mouse Gamer Redragon Paw3104 7200 DPI</t>
         </is>
       </c>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="39" t="inlineStr">
+      <c r="F30" s="28" t="n"/>
+      <c r="G30" s="31" t="inlineStr">
         <is>
           <t>Redragon</t>
         </is>
       </c>
-      <c r="H30" s="36" t="inlineStr">
+      <c r="H30" s="28" t="inlineStr">
         <is>
           <t>estoque baixo</t>
         </is>
@@ -1721,31 +1729,35 @@
     </row>
     <row r="31">
       <c r="A31" s="16" t="n"/>
-      <c r="B31" s="28" t="n">
+      <c r="B31" s="36" t="n">
         <v>30</v>
       </c>
-      <c r="C31" s="28" t="inlineStr">
+      <c r="C31" s="36" t="inlineStr">
         <is>
           <t>Mouse gamer sem fio</t>
         </is>
       </c>
-      <c r="D31" s="29" t="inlineStr">
+      <c r="D31" s="37" t="inlineStr">
         <is>
           <t>https://meli.la/241na5E</t>
         </is>
       </c>
-      <c r="E31" s="30" t="inlineStr">
+      <c r="E31" s="38" t="inlineStr">
         <is>
           <t>Mouse Gamer Redragon King Pro</t>
         </is>
       </c>
-      <c r="F31" s="28" t="n"/>
-      <c r="G31" s="31" t="inlineStr">
+      <c r="F31" s="36" t="n"/>
+      <c r="G31" s="39" t="inlineStr">
         <is>
           <t>Redragon</t>
         </is>
       </c>
-      <c r="H31" s="28" t="n"/>
+      <c r="H31" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>⬜</t>

</xml_diff>

<commit_message>
adicionando mouse com fio
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1638c87186bceadf/Desktop/OfertasTec/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_93A9383EEBD1B033BA28AB930C480551B8790B43" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55CA5FCD-1CCD-422A-B807-540CC12946D0}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_93A9383EEBA1B11C24EAF462A72A0351B8790B92" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA84F889-8952-4C31-985B-4A6260B183E9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="515">
   <si>
     <t>Validação</t>
   </si>
@@ -377,6 +377,9 @@
     <t>https://meli.la/321ZTMv</t>
   </si>
   <si>
+    <t>Mouse Gamer M711 Cobra Chroma Redragon Com fio Para Jogos 12.400 DPI Com Led RGB Preto</t>
+  </si>
+  <si>
     <t>https://meli.la/2nikVNt</t>
   </si>
   <si>
@@ -410,6 +413,9 @@
     <t>https://meli.la/23wdZ7w</t>
   </si>
   <si>
+    <t>Mouse Gamer 6 Botões 12.800 Dpi Sensor Instantâneo Kp-mu026</t>
+  </si>
+  <si>
     <t>https://meli.la/15mY31Y</t>
   </si>
   <si>
@@ -1563,12 +1569,6 @@
   </si>
   <si>
     <t>Vou usar os dados pra atualizar o site automaticamente.</t>
-  </si>
-  <si>
-    <t>Mouse Gamer M711 Cobra Chroma Redragon Com fio Para Jogos 12.400 DPI Com Led RGB Preto</t>
-  </si>
-  <si>
-    <t>Mouse Gamer 6 Botões 12.800 Dpi Sensor Instantâneo Kp-mu026</t>
   </si>
 </sst>
 </file>
@@ -2533,7 +2533,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16"/>
       <c r="B15" s="28">
         <v>14</v>
@@ -3208,7 +3208,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="16"/>
       <c r="B44" s="28">
         <v>43</v>
@@ -3220,7 +3220,7 @@
         <v>116</v>
       </c>
       <c r="E44" s="30" t="s">
-        <v>513</v>
+        <v>117</v>
       </c>
       <c r="F44" s="28"/>
       <c r="G44" s="28"/>
@@ -3229,7 +3229,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="16"/>
       <c r="B45" s="28">
         <v>44</v>
@@ -3238,21 +3238,21 @@
         <v>115</v>
       </c>
       <c r="D45" s="29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E45" s="30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F45" s="28"/>
       <c r="G45" s="28" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H45" s="28"/>
       <c r="I45" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="16"/>
       <c r="B46" s="28">
         <v>45</v>
@@ -3261,10 +3261,10 @@
         <v>115</v>
       </c>
       <c r="D46" s="29" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E46" s="30" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F46" s="28"/>
       <c r="G46" s="31" t="s">
@@ -3275,7 +3275,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="36">
         <v>46</v>
@@ -3284,10 +3284,10 @@
         <v>115</v>
       </c>
       <c r="D47" s="37" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E47" s="38" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F47" s="36"/>
       <c r="G47" s="39" t="s">
@@ -3300,7 +3300,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="16"/>
       <c r="B48" s="36">
         <v>47</v>
@@ -3309,14 +3309,14 @@
         <v>115</v>
       </c>
       <c r="D48" s="37" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E48" s="38" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F48" s="36"/>
       <c r="G48" s="36" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H48" s="36" t="s">
         <v>53</v>
@@ -3325,7 +3325,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="36">
         <v>48</v>
@@ -3334,10 +3334,10 @@
         <v>115</v>
       </c>
       <c r="D49" s="37" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E49" s="38" t="s">
-        <v>514</v>
+        <v>129</v>
       </c>
       <c r="F49" s="36"/>
       <c r="G49" s="36"/>
@@ -3348,7 +3348,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="16"/>
       <c r="B50" s="28">
         <v>49</v>
@@ -3357,21 +3357,21 @@
         <v>115</v>
       </c>
       <c r="D50" s="29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F50" s="28"/>
       <c r="G50" s="28" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H50" s="28"/>
       <c r="I50" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="16"/>
       <c r="B51" s="28">
         <v>50</v>
@@ -3380,10 +3380,10 @@
         <v>115</v>
       </c>
       <c r="D51" s="29" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E51" s="30" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F51" s="28"/>
       <c r="G51" s="31" t="s">
@@ -3394,7 +3394,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="16"/>
       <c r="B52" s="36">
         <v>51</v>
@@ -3403,14 +3403,14 @@
         <v>115</v>
       </c>
       <c r="D52" s="37" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E52" s="38" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F52" s="36"/>
       <c r="G52" s="39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H52" s="36" t="s">
         <v>53</v>
@@ -3419,7 +3419,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="16"/>
       <c r="B53" s="28">
         <v>52</v>
@@ -3428,21 +3428,21 @@
         <v>115</v>
       </c>
       <c r="D53" s="29" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E53" s="30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F53" s="28"/>
       <c r="G53" s="31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H53" s="28"/>
       <c r="I53" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="16"/>
       <c r="B54" s="28">
         <v>53</v>
@@ -3451,21 +3451,21 @@
         <v>115</v>
       </c>
       <c r="D54" s="29" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E54" s="30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F54" s="28"/>
       <c r="G54" s="31" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H54" s="28"/>
       <c r="I54" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="16"/>
       <c r="B55" s="36">
         <v>54</v>
@@ -3474,10 +3474,10 @@
         <v>115</v>
       </c>
       <c r="D55" s="37" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E55" s="38" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F55" s="36"/>
       <c r="G55" s="39" t="s">
@@ -3490,7 +3490,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="16"/>
       <c r="B56" s="36">
         <v>55</v>
@@ -3499,10 +3499,10 @@
         <v>115</v>
       </c>
       <c r="D56" s="37" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E56" s="38" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F56" s="36"/>
       <c r="G56" s="39" t="s">
@@ -3515,111 +3515,113 @@
         <v>13</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="16"/>
-      <c r="B57" s="28">
+      <c r="B57" s="36">
         <v>56</v>
       </c>
-      <c r="C57" s="28" t="s">
-        <v>144</v>
-      </c>
-      <c r="D57" s="29" t="s">
-        <v>145</v>
-      </c>
-      <c r="E57" s="30" t="s">
+      <c r="C57" s="36" t="s">
         <v>146</v>
       </c>
-      <c r="F57" s="28"/>
-      <c r="G57" s="31" t="s">
+      <c r="D57" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="E57" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="F57" s="36"/>
+      <c r="G57" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="H57" s="28"/>
+      <c r="H57" s="36" t="s">
+        <v>53</v>
+      </c>
       <c r="I57" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="16"/>
       <c r="B58" s="28">
         <v>57</v>
       </c>
       <c r="C58" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D58" s="29" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E58" s="30" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F58" s="28"/>
       <c r="G58" s="31" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H58" s="28"/>
       <c r="I58" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="16"/>
       <c r="B59" s="28">
         <v>58</v>
       </c>
       <c r="C59" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D59" s="29" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E59" s="30" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F59" s="28"/>
       <c r="G59" s="31" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H59" s="28"/>
       <c r="I59" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="16"/>
       <c r="B60" s="28">
         <v>59</v>
       </c>
       <c r="C60" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D60" s="29" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E60" s="30" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F60" s="28"/>
       <c r="G60" s="31" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H60" s="28"/>
       <c r="I60" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="16"/>
       <c r="B61" s="28">
         <v>60</v>
       </c>
       <c r="C61" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D61" s="29" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E61" s="30" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F61" s="28"/>
       <c r="G61" s="31" t="s">
@@ -3630,19 +3632,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="16"/>
       <c r="B62" s="28">
         <v>61</v>
       </c>
       <c r="C62" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D62" s="29" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E62" s="30" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F62" s="28"/>
       <c r="G62" s="31" t="s">
@@ -3653,16 +3655,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="54">
         <v>62</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="3"/>
@@ -3672,19 +3674,19 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="16"/>
       <c r="B64" s="28">
         <v>63</v>
       </c>
       <c r="C64" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D64" s="29" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E64" s="30" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F64" s="28"/>
       <c r="G64" s="31" t="s">
@@ -3695,46 +3697,46 @@
         <v>13</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
-      <c r="B65" s="54">
+      <c r="B65" s="28">
         <v>64</v>
       </c>
-      <c r="C65" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="F65" s="3"/>
-      <c r="G65" s="18" t="s">
+      <c r="C65" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="D65" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="H65" s="3"/>
+      <c r="E65" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="F65" s="28"/>
+      <c r="G65" s="31" t="s">
+        <v>167</v>
+      </c>
+      <c r="H65" s="28"/>
       <c r="I65" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="16"/>
       <c r="B66" s="28">
         <v>65</v>
       </c>
       <c r="C66" s="28" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D66" s="29" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E66" s="30" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F66" s="28"/>
       <c r="G66" s="31" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H66" s="28"/>
       <c r="I66" t="s">
@@ -3747,13 +3749,13 @@
         <v>66</v>
       </c>
       <c r="C67" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D67" s="29" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E67" s="30" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F67" s="28"/>
       <c r="G67" s="28" t="s">
@@ -3770,13 +3772,13 @@
         <v>67</v>
       </c>
       <c r="C68" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D68" s="29" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F68" s="28"/>
       <c r="G68" s="31" t="s">
@@ -3793,17 +3795,17 @@
         <v>68</v>
       </c>
       <c r="C69" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D69" s="29" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E69" s="30" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F69" s="28"/>
       <c r="G69" s="31" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H69" s="28"/>
       <c r="I69" t="s">
@@ -3816,17 +3818,17 @@
         <v>69</v>
       </c>
       <c r="C70" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D70" s="29" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E70" s="30" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F70" s="28"/>
       <c r="G70" s="31" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H70" s="28"/>
       <c r="I70" t="s">
@@ -3839,10 +3841,10 @@
         <v>70</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E71" s="6"/>
       <c r="F71" s="3"/>
@@ -3858,13 +3860,13 @@
         <v>71</v>
       </c>
       <c r="C72" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D72" s="29" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E72" s="30" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F72" s="28"/>
       <c r="G72" s="31" t="s">
@@ -3881,17 +3883,17 @@
         <v>72</v>
       </c>
       <c r="C73" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D73" s="29" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="E73" s="30" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F73" s="28"/>
       <c r="G73" s="31" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H73" s="28"/>
       <c r="I73" t="s">
@@ -3904,13 +3906,13 @@
         <v>73</v>
       </c>
       <c r="C74" s="28" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D74" s="29" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E74" s="30" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F74" s="28"/>
       <c r="G74" s="31" t="s">
@@ -3927,17 +3929,17 @@
         <v>74</v>
       </c>
       <c r="C75" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D75" s="29" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E75" s="30" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F75" s="28"/>
       <c r="G75" s="31" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H75" s="28"/>
       <c r="I75" t="s">
@@ -3949,10 +3951,10 @@
         <v>75</v>
       </c>
       <c r="C76" s="36" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D76" s="37" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E76" s="38"/>
       <c r="F76" s="36"/>
@@ -3970,17 +3972,17 @@
         <v>76</v>
       </c>
       <c r="C77" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D77" s="29" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E77" s="30" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F77" s="28"/>
       <c r="G77" s="31" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H77" s="28"/>
       <c r="I77" t="s">
@@ -3993,17 +3995,17 @@
         <v>77</v>
       </c>
       <c r="C78" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D78" s="29" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E78" s="30" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F78" s="28"/>
       <c r="G78" s="31" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H78" s="28"/>
       <c r="I78" t="s">
@@ -4016,17 +4018,17 @@
         <v>78</v>
       </c>
       <c r="C79" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D79" s="29" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E79" s="30" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F79" s="28"/>
       <c r="G79" s="31" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H79" s="28"/>
       <c r="I79" t="s">
@@ -4039,10 +4041,10 @@
         <v>79</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E80" s="6"/>
       <c r="F80" s="3"/>
@@ -4058,13 +4060,13 @@
         <v>80</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E81" s="6" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
@@ -4079,17 +4081,17 @@
         <v>81</v>
       </c>
       <c r="C82" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D82" s="29" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E82" s="30" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F82" s="28"/>
       <c r="G82" s="31" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="H82" s="28"/>
       <c r="I82" t="s">
@@ -4102,17 +4104,17 @@
         <v>82</v>
       </c>
       <c r="C83" s="32" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D83" s="33" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E83" s="34" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F83" s="32"/>
       <c r="G83" s="35" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H83" s="32" t="s">
         <v>35</v>
@@ -4127,17 +4129,17 @@
         <v>83</v>
       </c>
       <c r="C84" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D84" s="29" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E84" s="30" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F84" s="28"/>
       <c r="G84" s="31" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="H84" s="28"/>
       <c r="I84" t="s">
@@ -4150,17 +4152,17 @@
         <v>84</v>
       </c>
       <c r="C85" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D85" s="29" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E85" s="30" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F85" s="28"/>
       <c r="G85" s="31" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="H85" s="28"/>
       <c r="I85" t="s">
@@ -4173,13 +4175,13 @@
         <v>85</v>
       </c>
       <c r="C86" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D86" s="29" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E86" s="30" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F86" s="28"/>
       <c r="G86" s="31" t="s">
@@ -4196,13 +4198,13 @@
         <v>86</v>
       </c>
       <c r="C87" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D87" s="29" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E87" s="30" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F87" s="28"/>
       <c r="G87" s="31" t="s">
@@ -4219,17 +4221,17 @@
         <v>87</v>
       </c>
       <c r="C88" s="28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D88" s="29" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E88" s="30" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F88" s="28"/>
       <c r="G88" s="31" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H88" s="28"/>
       <c r="I88" t="s">
@@ -4242,17 +4244,17 @@
         <v>88</v>
       </c>
       <c r="C89" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D89" s="29" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E89" s="30" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F89" s="28"/>
       <c r="G89" s="31" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H89" s="28"/>
       <c r="I89" t="s">
@@ -4265,17 +4267,17 @@
         <v>89</v>
       </c>
       <c r="C90" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D90" s="29" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E90" s="30" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F90" s="28"/>
       <c r="G90" s="31" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="H90" s="28"/>
       <c r="I90" t="s">
@@ -4288,17 +4290,17 @@
         <v>90</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D91" s="29" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E91" s="30" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F91" s="28"/>
       <c r="G91" s="31" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H91" s="28"/>
       <c r="I91" t="s">
@@ -4311,17 +4313,17 @@
         <v>91</v>
       </c>
       <c r="C92" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D92" s="29" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="E92" s="30" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F92" s="28"/>
       <c r="G92" s="31" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H92" s="28"/>
       <c r="I92" t="s">
@@ -4334,10 +4336,10 @@
         <v>92</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E93" s="6"/>
       <c r="F93" s="3"/>
@@ -4353,13 +4355,13 @@
         <v>93</v>
       </c>
       <c r="C94" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="E94" s="30" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F94" s="28"/>
       <c r="G94" s="31" t="s">
@@ -4376,17 +4378,17 @@
         <v>94</v>
       </c>
       <c r="C95" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D95" s="29" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E95" s="30" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F95" s="28"/>
       <c r="G95" s="31" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="H95" s="28"/>
       <c r="I95" t="s">
@@ -4399,17 +4401,17 @@
         <v>95</v>
       </c>
       <c r="C96" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D96" s="29" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E96" s="30" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F96" s="28"/>
       <c r="G96" s="31" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H96" s="28"/>
       <c r="I96" t="s">
@@ -4422,17 +4424,17 @@
         <v>96</v>
       </c>
       <c r="C97" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D97" s="29" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E97" s="30" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="F97" s="28"/>
       <c r="G97" s="31" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="H97" s="28"/>
       <c r="I97" t="s">
@@ -4445,10 +4447,10 @@
         <v>97</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E98" s="6"/>
       <c r="F98" s="3"/>
@@ -4464,10 +4466,10 @@
         <v>98</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="E99" s="6"/>
       <c r="F99" s="3"/>
@@ -4483,17 +4485,17 @@
         <v>99</v>
       </c>
       <c r="C100" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D100" s="29" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E100" s="30" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F100" s="28"/>
       <c r="G100" s="31" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="H100" s="28"/>
       <c r="I100" t="s">
@@ -4506,17 +4508,17 @@
         <v>100</v>
       </c>
       <c r="C101" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D101" s="29" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E101" s="30" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F101" s="28"/>
       <c r="G101" s="31" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H101" s="28"/>
       <c r="I101" t="s">
@@ -4529,17 +4531,17 @@
         <v>101</v>
       </c>
       <c r="C102" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D102" s="29" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E102" s="30" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F102" s="28"/>
       <c r="G102" s="31" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H102" s="28"/>
       <c r="I102" t="s">
@@ -4552,17 +4554,17 @@
         <v>102</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="18" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H103" s="3"/>
       <c r="I103" s="3" t="s">
@@ -4575,17 +4577,17 @@
         <v>103</v>
       </c>
       <c r="C104" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D104" s="29" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E104" s="30" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F104" s="28"/>
       <c r="G104" s="31" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H104" s="28"/>
       <c r="I104" t="s">
@@ -4598,10 +4600,10 @@
         <v>104</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E105" s="6"/>
       <c r="F105" s="3"/>
@@ -4617,17 +4619,17 @@
         <v>105</v>
       </c>
       <c r="C106" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D106" s="29" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E106" s="30" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F106" s="28"/>
       <c r="G106" s="31" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="H106" s="28"/>
       <c r="I106" t="s">
@@ -4640,17 +4642,17 @@
         <v>106</v>
       </c>
       <c r="C107" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D107" s="29" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E107" s="30" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="F107" s="28"/>
       <c r="G107" s="31" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H107" s="28"/>
       <c r="I107" t="s">
@@ -4663,17 +4665,17 @@
         <v>107</v>
       </c>
       <c r="C108" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D108" s="29" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E108" s="30" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="F108" s="28"/>
       <c r="G108" s="31" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="H108" s="28"/>
       <c r="I108" t="s">
@@ -4686,10 +4688,10 @@
         <v>108</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E109" s="6"/>
       <c r="F109" s="3"/>
@@ -4705,17 +4707,17 @@
         <v>109</v>
       </c>
       <c r="C110" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D110" s="29" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="E110" s="30" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="F110" s="28"/>
       <c r="G110" s="31" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="H110" s="28"/>
       <c r="I110" t="s">
@@ -4728,17 +4730,17 @@
         <v>110</v>
       </c>
       <c r="C111" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D111" s="29" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E111" s="30" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="F111" s="28"/>
       <c r="G111" s="31" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="H111" s="28"/>
       <c r="I111" t="s">
@@ -4751,17 +4753,17 @@
         <v>111</v>
       </c>
       <c r="C112" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D112" s="29" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E112" s="30" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="F112" s="28"/>
       <c r="G112" s="31" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="H112" s="28"/>
       <c r="I112" t="s">
@@ -4774,10 +4776,10 @@
         <v>112</v>
       </c>
       <c r="C113" s="9" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E113" s="11"/>
       <c r="F113" s="9"/>
@@ -4793,17 +4795,17 @@
         <v>113</v>
       </c>
       <c r="C114" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D114" s="29" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="E114" s="30" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F114" s="28"/>
       <c r="G114" s="31" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="H114" s="28"/>
       <c r="I114" t="s">
@@ -4816,17 +4818,17 @@
         <v>114</v>
       </c>
       <c r="C115" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D115" s="29" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E115" s="30" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F115" s="28"/>
       <c r="G115" s="31" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H115" s="28"/>
       <c r="I115" t="s">
@@ -4839,17 +4841,17 @@
         <v>115</v>
       </c>
       <c r="C116" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D116" s="29" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E116" s="30" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F116" s="28"/>
       <c r="G116" s="28" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H116" s="28"/>
       <c r="I116" t="s">
@@ -4862,17 +4864,17 @@
         <v>116</v>
       </c>
       <c r="C117" s="28" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D117" s="29" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E117" s="30" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="F117" s="28"/>
       <c r="G117" s="31" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H117" s="28"/>
       <c r="I117" t="s">
@@ -4885,10 +4887,10 @@
         <v>117</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="E118" s="6"/>
       <c r="F118" s="3"/>
@@ -4904,13 +4906,13 @@
         <v>118</v>
       </c>
       <c r="C119" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D119" s="29" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E119" s="30" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F119" s="28"/>
       <c r="G119" s="31" t="s">
@@ -4927,17 +4929,17 @@
         <v>119</v>
       </c>
       <c r="C120" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D120" s="29" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E120" s="30" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F120" s="28"/>
       <c r="G120" s="31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H120" s="28"/>
       <c r="I120" t="s">
@@ -4950,13 +4952,13 @@
         <v>120</v>
       </c>
       <c r="C121" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D121" s="29" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E121" s="30" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F121" s="28"/>
       <c r="G121" s="31" t="s">
@@ -4973,10 +4975,10 @@
         <v>121</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="E122" s="6"/>
       <c r="F122" s="3"/>
@@ -4992,17 +4994,17 @@
         <v>122</v>
       </c>
       <c r="C123" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D123" s="29" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E123" s="30" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="F123" s="28"/>
       <c r="G123" s="31" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H123" s="28"/>
       <c r="I123" t="s">
@@ -5015,17 +5017,17 @@
         <v>123</v>
       </c>
       <c r="C124" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D124" s="29" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E124" s="30" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F124" s="28"/>
       <c r="G124" s="28" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="H124" s="28"/>
       <c r="I124" t="s">
@@ -5038,17 +5040,17 @@
         <v>124</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D125" s="13" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E125" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="F125" s="12"/>
       <c r="G125" s="15" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H125" s="12"/>
       <c r="I125" s="12" t="s">
@@ -5061,13 +5063,13 @@
         <v>125</v>
       </c>
       <c r="C126" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D126" s="29" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="E126" s="30" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F126" s="28"/>
       <c r="G126" s="28" t="s">
@@ -5084,17 +5086,17 @@
         <v>126</v>
       </c>
       <c r="C127" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D127" s="29" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="E127" s="30" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F127" s="28"/>
       <c r="G127" s="31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H127" s="28"/>
       <c r="I127" t="s">
@@ -5107,17 +5109,17 @@
         <v>127</v>
       </c>
       <c r="C128" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D128" s="29" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="E128" s="30" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F128" s="28"/>
       <c r="G128" s="28" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H128" s="28"/>
       <c r="I128" t="s">
@@ -5130,17 +5132,17 @@
         <v>128</v>
       </c>
       <c r="C129" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D129" s="29" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E129" s="30" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F129" s="28"/>
       <c r="G129" s="31" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="H129" s="28"/>
       <c r="I129" t="s">
@@ -5153,17 +5155,17 @@
         <v>129</v>
       </c>
       <c r="C130" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D130" s="29" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E130" s="28" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F130" s="28"/>
       <c r="G130" s="31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H130" s="28"/>
       <c r="I130" t="s">
@@ -5176,17 +5178,17 @@
         <v>130</v>
       </c>
       <c r="C131" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D131" s="29" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E131" s="28" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="F131" s="28"/>
       <c r="G131" s="31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H131" s="28"/>
       <c r="I131" t="s">
@@ -5199,13 +5201,13 @@
         <v>131</v>
       </c>
       <c r="C132" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D132" s="29" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E132" s="30" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F132" s="28"/>
       <c r="G132" s="31" t="s">
@@ -5222,17 +5224,17 @@
         <v>132</v>
       </c>
       <c r="C133" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D133" s="29" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E133" s="30" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F133" s="28"/>
       <c r="G133" s="31" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="H133" s="28"/>
       <c r="I133" t="s">
@@ -5245,17 +5247,17 @@
         <v>133</v>
       </c>
       <c r="C134" s="28" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D134" s="29" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E134" s="30" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F134" s="28"/>
       <c r="G134" s="31" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="H134" s="28"/>
       <c r="I134" t="s">
@@ -5268,17 +5270,17 @@
         <v>134</v>
       </c>
       <c r="C135" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D135" s="29" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E135" s="30" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F135" s="28"/>
       <c r="G135" s="31" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="H135" s="28"/>
       <c r="I135" t="s">
@@ -5291,17 +5293,17 @@
         <v>135</v>
       </c>
       <c r="C136" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D136" s="29" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E136" s="30" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F136" s="28"/>
       <c r="G136" s="31" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H136" s="28"/>
       <c r="I136" t="s">
@@ -5314,17 +5316,17 @@
         <v>136</v>
       </c>
       <c r="C137" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D137" s="29" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E137" s="30" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F137" s="28"/>
       <c r="G137" s="31" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="H137" s="28"/>
       <c r="I137" t="s">
@@ -5337,17 +5339,17 @@
         <v>137</v>
       </c>
       <c r="C138" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D138" s="29" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E138" s="30" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F138" s="28"/>
       <c r="G138" s="31" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H138" s="28"/>
       <c r="I138" t="s">
@@ -5360,17 +5362,17 @@
         <v>138</v>
       </c>
       <c r="C139" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D139" s="29" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="E139" s="30" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="F139" s="28"/>
       <c r="G139" s="31" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="H139" s="28"/>
       <c r="I139" t="s">
@@ -5383,17 +5385,17 @@
         <v>139</v>
       </c>
       <c r="C140" s="28" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D140" s="29" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E140" s="30" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="F140" s="28"/>
       <c r="G140" s="31" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="H140" s="28"/>
       <c r="I140" t="s">
@@ -5406,17 +5408,17 @@
         <v>140</v>
       </c>
       <c r="C141" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D141" s="40" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E141" s="30" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F141" s="28"/>
       <c r="G141" s="31" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="H141" s="28"/>
     </row>
@@ -5426,17 +5428,17 @@
         <v>141</v>
       </c>
       <c r="C142" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D142" s="40" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E142" s="30" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="F142" s="28"/>
       <c r="G142" s="31" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="H142" s="28"/>
     </row>
@@ -5446,17 +5448,17 @@
         <v>142</v>
       </c>
       <c r="C143" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D143" s="40" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E143" s="30" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F143" s="28"/>
       <c r="G143" s="31" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="H143" s="28"/>
     </row>
@@ -5466,13 +5468,13 @@
         <v>143</v>
       </c>
       <c r="C144" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D144" s="40" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="E144" s="30" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="F144" s="28"/>
       <c r="G144" s="31" t="s">
@@ -5486,17 +5488,17 @@
         <v>144</v>
       </c>
       <c r="C145" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D145" s="42" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E145" s="38" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F145" s="36"/>
       <c r="G145" s="39" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="H145" s="36" t="s">
         <v>53</v>
@@ -5508,17 +5510,17 @@
         <v>145</v>
       </c>
       <c r="C146" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D146" s="40" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="E146" s="30" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="F146" s="28"/>
       <c r="G146" s="31" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="H146" s="28"/>
     </row>
@@ -5528,17 +5530,17 @@
         <v>146</v>
       </c>
       <c r="C147" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D147" s="40" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="E147" s="30" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="F147" s="28"/>
       <c r="G147" s="31" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="H147" s="28"/>
     </row>
@@ -5548,17 +5550,17 @@
         <v>147</v>
       </c>
       <c r="C148" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D148" s="40" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E148" s="30" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F148" s="28"/>
       <c r="G148" s="31" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="H148" s="28"/>
     </row>
@@ -5568,13 +5570,13 @@
         <v>148</v>
       </c>
       <c r="C149" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D149" s="40" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="E149" s="30" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="F149" s="28"/>
       <c r="G149" s="31" t="s">
@@ -5588,17 +5590,17 @@
         <v>149</v>
       </c>
       <c r="C150" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D150" s="42" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E150" s="38" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F150" s="36"/>
       <c r="G150" s="39" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="H150" s="36" t="s">
         <v>53</v>
@@ -5609,17 +5611,17 @@
         <v>150</v>
       </c>
       <c r="C151" s="47" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D151" s="53" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E151" s="49" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="F151" s="47"/>
       <c r="G151" s="50" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="H151" s="47"/>
     </row>
@@ -5629,17 +5631,17 @@
         <v>151</v>
       </c>
       <c r="C152" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D152" s="40" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E152" s="30" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="F152" s="30"/>
       <c r="G152" s="31" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="H152" s="28"/>
     </row>
@@ -5649,17 +5651,17 @@
         <v>152</v>
       </c>
       <c r="C153" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D153" s="40" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="E153" s="30" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F153" s="43"/>
       <c r="G153" s="31" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="H153" s="28"/>
     </row>
@@ -5669,17 +5671,17 @@
         <v>153</v>
       </c>
       <c r="C154" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D154" s="40" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E154" s="30" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F154" s="30"/>
       <c r="G154" s="31" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="H154" s="28"/>
     </row>
@@ -5689,17 +5691,17 @@
         <v>154</v>
       </c>
       <c r="C155" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D155" s="42" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E155" s="38" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F155" s="44"/>
       <c r="G155" s="39" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="H155" s="36" t="s">
         <v>53</v>
@@ -5711,13 +5713,13 @@
         <v>155</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D156" s="8" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="E156" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="F156" s="6"/>
       <c r="G156" s="3"/>
@@ -5730,13 +5732,13 @@
         <v>156</v>
       </c>
       <c r="C157" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D157" s="40" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E157" s="30" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F157" s="28"/>
       <c r="G157" s="28"/>
@@ -5747,13 +5749,13 @@
         <v>157</v>
       </c>
       <c r="C158" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D158" s="40" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E158" s="30" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="F158" s="28"/>
       <c r="G158" s="28"/>
@@ -5764,13 +5766,13 @@
         <v>158</v>
       </c>
       <c r="C159" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D159" s="42" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="E159" s="38" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="F159" s="36"/>
       <c r="G159" s="36"/>
@@ -5783,13 +5785,13 @@
         <v>159</v>
       </c>
       <c r="C160" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D160" s="42" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E160" s="38" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F160" s="36"/>
       <c r="G160" s="36"/>
@@ -5802,13 +5804,13 @@
         <v>160</v>
       </c>
       <c r="C161" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D161" s="40" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="E161" s="30" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="F161" s="30"/>
       <c r="G161" s="30"/>
@@ -5820,13 +5822,13 @@
         <v>161</v>
       </c>
       <c r="C162" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D162" s="42" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E162" s="38" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F162" s="38"/>
       <c r="G162" s="38"/>
@@ -5859,13 +5861,13 @@
         <v>162</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D163" s="25" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="E163" s="6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="F163" s="6"/>
       <c r="G163" s="6"/>
@@ -5896,13 +5898,13 @@
         <v>163</v>
       </c>
       <c r="C164" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D164" s="42" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E164" s="38" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F164" s="38"/>
       <c r="G164" s="38"/>
@@ -5934,13 +5936,13 @@
         <v>164</v>
       </c>
       <c r="C165" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D165" s="40" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="E165" s="30" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F165" s="30"/>
       <c r="G165" s="30"/>
@@ -5970,13 +5972,13 @@
         <v>165</v>
       </c>
       <c r="C166" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D166" s="40" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E166" s="30" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F166" s="30"/>
       <c r="G166" s="30"/>
@@ -6006,13 +6008,13 @@
         <v>166</v>
       </c>
       <c r="C167" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D167" s="40" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E167" s="30" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F167" s="30"/>
       <c r="G167" s="30"/>
@@ -6042,13 +6044,13 @@
         <v>167</v>
       </c>
       <c r="C168" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D168" s="40" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="E168" s="30" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="F168" s="30"/>
       <c r="G168" s="30"/>
@@ -6078,13 +6080,13 @@
         <v>168</v>
       </c>
       <c r="C169" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D169" s="42" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E169" s="38" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F169" s="38"/>
       <c r="G169" s="38"/>
@@ -6116,13 +6118,13 @@
         <v>169</v>
       </c>
       <c r="C170" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D170" s="40" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="E170" s="30" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="F170" s="30"/>
       <c r="G170" s="30"/>
@@ -6152,13 +6154,13 @@
         <v>170</v>
       </c>
       <c r="C171" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D171" s="40" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E171" s="30" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F171" s="30"/>
       <c r="G171" s="30"/>
@@ -6188,13 +6190,13 @@
         <v>171</v>
       </c>
       <c r="C172" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D172" s="42" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="E172" s="38" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F172" s="38"/>
       <c r="G172" s="38"/>
@@ -6226,13 +6228,13 @@
         <v>172</v>
       </c>
       <c r="C173" s="36" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D173" s="42" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E173" s="38" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F173" s="38"/>
       <c r="G173" s="38"/>
@@ -6264,13 +6266,13 @@
         <v>173</v>
       </c>
       <c r="C174" s="32" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D174" s="45" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="E174" s="34" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="F174" s="34"/>
       <c r="G174" s="34"/>
@@ -6302,13 +6304,13 @@
         <v>174</v>
       </c>
       <c r="C175" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D175" s="40" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E175" s="30" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F175" s="30"/>
       <c r="G175" s="30"/>
@@ -6338,13 +6340,13 @@
         <v>175</v>
       </c>
       <c r="C176" s="28" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D176" s="40" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="E176" s="30" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="F176" s="30"/>
       <c r="G176" s="30"/>
@@ -6374,13 +6376,13 @@
         <v>176</v>
       </c>
       <c r="C177" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D177" s="40" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E177" s="30" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F177" s="30"/>
       <c r="G177" s="30"/>
@@ -6410,13 +6412,13 @@
         <v>177</v>
       </c>
       <c r="C178" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D178" s="40" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="E178" s="30" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="F178" s="30"/>
       <c r="G178" s="30"/>
@@ -6446,13 +6448,13 @@
         <v>178</v>
       </c>
       <c r="C179" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D179" s="40" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="E179" s="30" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F179" s="30"/>
       <c r="G179" s="30"/>
@@ -6482,13 +6484,13 @@
         <v>179</v>
       </c>
       <c r="C180" s="36" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D180" s="42" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E180" s="38" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F180" s="38"/>
       <c r="G180" s="38"/>
@@ -6520,13 +6522,13 @@
         <v>180</v>
       </c>
       <c r="C181" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D181" s="40" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="E181" s="30" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F181" s="30"/>
       <c r="G181" s="30"/>
@@ -6556,13 +6558,13 @@
         <v>181</v>
       </c>
       <c r="C182" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D182" s="40" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E182" s="30" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F182" s="30"/>
       <c r="G182" s="30"/>
@@ -6592,13 +6594,13 @@
         <v>182</v>
       </c>
       <c r="C183" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D183" s="40" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="E183" s="30" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="F183" s="30"/>
       <c r="G183" s="30"/>
@@ -6628,13 +6630,13 @@
         <v>183</v>
       </c>
       <c r="C184" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D184" s="40" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="E184" s="30" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F184" s="30"/>
       <c r="G184" s="30"/>
@@ -6664,13 +6666,13 @@
         <v>184</v>
       </c>
       <c r="C185" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D185" s="40" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E185" s="30" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F185" s="30"/>
       <c r="G185" s="30"/>
@@ -6700,13 +6702,13 @@
         <v>185</v>
       </c>
       <c r="C186" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D186" s="40" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E186" s="30" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F186" s="30"/>
       <c r="G186" s="30"/>
@@ -6736,13 +6738,13 @@
         <v>186</v>
       </c>
       <c r="C187" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D187" s="40" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="E187" s="30" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="F187" s="30"/>
       <c r="G187" s="30"/>
@@ -6772,13 +6774,13 @@
         <v>187</v>
       </c>
       <c r="C188" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D188" s="40" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="E188" s="30" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F188" s="30"/>
       <c r="G188" s="30"/>
@@ -6808,13 +6810,13 @@
         <v>188</v>
       </c>
       <c r="C189" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D189" s="40" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E189" s="30" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F189" s="30"/>
       <c r="G189" s="30"/>
@@ -6844,13 +6846,13 @@
         <v>189</v>
       </c>
       <c r="C190" s="28" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D190" s="40" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E190" s="30" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F190" s="30"/>
       <c r="G190" s="30"/>
@@ -6880,13 +6882,13 @@
         <v>190</v>
       </c>
       <c r="C191" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D191" s="40" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E191" s="30" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F191" s="30"/>
       <c r="G191" s="30"/>
@@ -6916,13 +6918,13 @@
         <v>191</v>
       </c>
       <c r="C192" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D192" s="40" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E192" s="30" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F192" s="28"/>
       <c r="G192" s="28"/>
@@ -6951,13 +6953,13 @@
         <v>192</v>
       </c>
       <c r="C193" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D193" s="40" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E193" s="30" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F193" s="28"/>
       <c r="G193" s="28"/>
@@ -6968,13 +6970,13 @@
         <v>193</v>
       </c>
       <c r="C194" s="36" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D194" s="42" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E194" s="38" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F194" s="36"/>
       <c r="G194" s="36"/>
@@ -6987,13 +6989,13 @@
         <v>194</v>
       </c>
       <c r="C195" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D195" s="40" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="E195" s="30" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="F195" s="28"/>
       <c r="G195" s="28"/>
@@ -7004,13 +7006,13 @@
         <v>195</v>
       </c>
       <c r="C196" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D196" s="40" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E196" s="30" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="F196" s="28"/>
       <c r="G196" s="28"/>
@@ -7021,13 +7023,13 @@
         <v>196</v>
       </c>
       <c r="C197" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D197" s="40" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="E197" s="30" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="F197" s="28"/>
       <c r="G197" s="28"/>
@@ -7038,13 +7040,13 @@
         <v>197</v>
       </c>
       <c r="C198" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D198" s="40" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="E198" s="30" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F198" s="28"/>
       <c r="G198" s="28"/>
@@ -7055,13 +7057,13 @@
         <v>198</v>
       </c>
       <c r="C199" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D199" s="40" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E199" s="30" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F199" s="28"/>
       <c r="G199" s="28"/>
@@ -7072,13 +7074,13 @@
         <v>199</v>
       </c>
       <c r="C200" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D200" s="40" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="E200" s="30" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="F200" s="28"/>
       <c r="G200" s="28"/>
@@ -7089,13 +7091,13 @@
         <v>200</v>
       </c>
       <c r="C201" s="36" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D201" s="42" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="E201" s="38" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="F201" s="36"/>
       <c r="G201" s="36"/>
@@ -7108,13 +7110,13 @@
         <v>201</v>
       </c>
       <c r="C202" s="28" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D202" s="40" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="E202" s="30" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F202" s="28"/>
       <c r="G202" s="28"/>
@@ -7128,10 +7130,10 @@
         <v>9</v>
       </c>
       <c r="D203" s="57" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E203" s="58" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F203" s="54"/>
       <c r="G203" s="54"/>
@@ -7147,10 +7149,10 @@
         <v>9</v>
       </c>
       <c r="D204" s="40" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="E204" s="30" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="F204" s="28"/>
       <c r="G204" s="28"/>
@@ -7165,10 +7167,10 @@
         <v>9</v>
       </c>
       <c r="D205" s="40" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E205" s="30" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F205" s="28"/>
       <c r="G205" s="28"/>
@@ -7183,10 +7185,10 @@
         <v>9</v>
       </c>
       <c r="D206" s="40" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E206" s="30" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F206" s="28"/>
       <c r="G206" s="28"/>
@@ -7201,10 +7203,10 @@
         <v>9</v>
       </c>
       <c r="D207" s="40" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="E207" s="30" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="F207" s="28"/>
       <c r="G207" s="28"/>
@@ -7219,10 +7221,10 @@
         <v>9</v>
       </c>
       <c r="D208" s="40" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E208" s="30" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F208" s="28"/>
       <c r="G208" s="28"/>
@@ -7237,10 +7239,10 @@
         <v>9</v>
       </c>
       <c r="D209" s="42" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="E209" s="38" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F209" s="36"/>
       <c r="G209" s="36"/>
@@ -7257,10 +7259,10 @@
         <v>9</v>
       </c>
       <c r="D210" s="40" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E210" s="30" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F210" s="28"/>
       <c r="G210" s="28"/>
@@ -7275,10 +7277,10 @@
         <v>9</v>
       </c>
       <c r="D211" s="40" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="E211" s="30" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F211" s="28"/>
       <c r="G211" s="28"/>
@@ -7671,7 +7673,7 @@
   <autoFilter ref="A1:I253" xr:uid="{00000000-0009-0000-0000-000000000000}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Mouse gamer com fio"/>
+        <filter val="Teclado com fio"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -7901,92 +7903,92 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
colocando fone sem fio (bluetooth)
</commit_message>
<xml_diff>
--- a/Produtos_ml.xlsx
+++ b/Produtos_ml.xlsx
@@ -698,7 +698,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AA1974"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="6.7109375" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
     </row>
-    <row r="67">
+    <row r="67" hidden="1">
       <c r="A67" s="16" t="n"/>
       <c r="B67" s="36" t="n">
         <v>66</v>
@@ -2968,7 +2968,7 @@
         </is>
       </c>
     </row>
-    <row r="68">
+    <row r="68" hidden="1">
       <c r="A68" s="16" t="n"/>
       <c r="B68" s="28" t="n">
         <v>67</v>
@@ -3001,7 +3001,7 @@
         </is>
       </c>
     </row>
-    <row r="69">
+    <row r="69" hidden="1">
       <c r="A69" s="16" t="n"/>
       <c r="B69" s="32" t="n">
         <v>68</v>
@@ -3038,7 +3038,7 @@
         </is>
       </c>
     </row>
-    <row r="70">
+    <row r="70" hidden="1">
       <c r="A70" s="16" t="n"/>
       <c r="B70" s="36" t="n">
         <v>69</v>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
     </row>
-    <row r="71">
+    <row r="71" hidden="1">
       <c r="A71" s="3" t="n"/>
       <c r="B71" s="28" t="n">
         <v>70</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
     </row>
-    <row r="72">
+    <row r="72" hidden="1">
       <c r="A72" s="16" t="n"/>
       <c r="B72" s="28" t="n">
         <v>71</v>
@@ -3133,7 +3133,7 @@
         </is>
       </c>
     </row>
-    <row r="73">
+    <row r="73" hidden="1">
       <c r="A73" s="16" t="n"/>
       <c r="B73" s="28" t="n">
         <v>72</v>
@@ -3166,7 +3166,7 @@
         </is>
       </c>
     </row>
-    <row r="74">
+    <row r="74" hidden="1">
       <c r="A74" s="16" t="n"/>
       <c r="B74" s="28" t="n">
         <v>73</v>
@@ -3648,7 +3648,7 @@
         </is>
       </c>
     </row>
-    <row r="89" hidden="1">
+    <row r="89">
       <c r="A89" s="16" t="n"/>
       <c r="B89" s="28" t="n">
         <v>88</v>
@@ -3681,40 +3681,44 @@
         </is>
       </c>
     </row>
-    <row r="90" hidden="1">
+    <row r="90">
       <c r="A90" s="16" t="n"/>
-      <c r="B90" s="28" t="n">
+      <c r="B90" s="36" t="n">
         <v>89</v>
       </c>
-      <c r="C90" s="28" t="inlineStr">
+      <c r="C90" s="36" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D90" s="29" t="inlineStr">
+      <c r="D90" s="37" t="inlineStr">
         <is>
           <t>https://meli.la/1vyVnBY</t>
         </is>
       </c>
-      <c r="E90" s="30" t="inlineStr">
+      <c r="E90" s="38" t="inlineStr">
         <is>
           <t>Fones de ouvido Bluetooth esportivos sem fio Ipx7 5.3.650 mAh, Bluetooth 5.3, cancelamento de ruído Enc, tela LED, resistência à água IPX7, para negócios, entretenimento e corrida</t>
         </is>
       </c>
-      <c r="F90" s="28" t="n"/>
-      <c r="G90" s="31" t="inlineStr">
+      <c r="F90" s="36" t="n"/>
+      <c r="G90" s="39" t="inlineStr">
         <is>
           <t>MerttoBX28</t>
         </is>
       </c>
-      <c r="H90" s="28" t="n"/>
+      <c r="H90" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
       <c r="I90" t="inlineStr">
         <is>
           <t>⬜</t>
         </is>
       </c>
     </row>
-    <row r="91" hidden="1">
+    <row r="91">
       <c r="A91" s="16" t="n"/>
       <c r="B91" s="28" t="n">
         <v>90</v>
@@ -3747,7 +3751,7 @@
         </is>
       </c>
     </row>
-    <row r="92" hidden="1">
+    <row r="92">
       <c r="A92" s="16" t="n"/>
       <c r="B92" s="28" t="n">
         <v>91</v>
@@ -3780,7 +3784,7 @@
         </is>
       </c>
     </row>
-    <row r="93" hidden="1">
+    <row r="93">
       <c r="A93" s="3" t="n"/>
       <c r="B93" s="54" t="n">
         <v>92</v>
@@ -3805,7 +3809,7 @@
         </is>
       </c>
     </row>
-    <row r="94" hidden="1">
+    <row r="94">
       <c r="A94" s="16" t="n"/>
       <c r="B94" s="28" t="n">
         <v>93</v>
@@ -3838,7 +3842,7 @@
         </is>
       </c>
     </row>
-    <row r="95" hidden="1">
+    <row r="95">
       <c r="A95" s="16" t="n"/>
       <c r="B95" s="28" t="n">
         <v>94</v>
@@ -3871,40 +3875,44 @@
         </is>
       </c>
     </row>
-    <row r="96" hidden="1">
+    <row r="96">
       <c r="A96" s="16" t="n"/>
-      <c r="B96" s="28" t="n">
+      <c r="B96" s="36" t="n">
         <v>95</v>
       </c>
-      <c r="C96" s="28" t="inlineStr">
+      <c r="C96" s="36" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D96" s="29" t="inlineStr">
+      <c r="D96" s="37" t="inlineStr">
         <is>
           <t>https://meli.la/1G18uM3</t>
         </is>
       </c>
-      <c r="E96" s="30" t="inlineStr">
+      <c r="E96" s="38" t="inlineStr">
         <is>
           <t>Fone De Ouvido Bluetooth Jbl Tune Flex 2 Preto</t>
         </is>
       </c>
-      <c r="F96" s="28" t="n"/>
-      <c r="G96" s="31" t="inlineStr">
+      <c r="F96" s="36" t="n"/>
+      <c r="G96" s="39" t="inlineStr">
         <is>
           <t>JBL</t>
         </is>
       </c>
-      <c r="H96" s="28" t="n"/>
+      <c r="H96" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t>⬜</t>
         </is>
       </c>
     </row>
-    <row r="97" hidden="1">
+    <row r="97">
       <c r="A97" s="16" t="n"/>
       <c r="B97" s="28" t="n">
         <v>96</v>
@@ -3937,7 +3945,7 @@
         </is>
       </c>
     </row>
-    <row r="98" hidden="1">
+    <row r="98">
       <c r="A98" s="3" t="n"/>
       <c r="B98" s="54" t="n">
         <v>97</v>
@@ -3962,32 +3970,36 @@
         </is>
       </c>
     </row>
-    <row r="99" hidden="1">
+    <row r="99">
       <c r="A99" s="3" t="n"/>
-      <c r="B99" s="54" t="n">
+      <c r="B99" s="28" t="n">
         <v>98</v>
       </c>
-      <c r="C99" s="3" t="inlineStr">
+      <c r="C99" s="28" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D99" s="4" t="inlineStr">
+      <c r="D99" s="29" t="inlineStr">
         <is>
           <t>https://meli.la/2L2DTy9</t>
         </is>
       </c>
-      <c r="E99" s="6" t="n"/>
-      <c r="F99" s="3" t="n"/>
-      <c r="G99" s="3" t="n"/>
-      <c r="H99" s="3" t="n"/>
+      <c r="E99" s="30" t="inlineStr">
+        <is>
+          <t>Fone de Ouvido Bluetooth 5.4 soundcore P30i da Anker, Cancelamento de Ruído Adaptativo, Graves Poderosos, 45H de Reprodução, Estojo 2-em-1 com Suporte para Celular, IP54, Fone sem fio TWS, Branco</t>
+        </is>
+      </c>
+      <c r="F99" s="28" t="n"/>
+      <c r="G99" s="28" t="n"/>
+      <c r="H99" s="28" t="n"/>
       <c r="I99" s="3" t="inlineStr">
         <is>
           <t>⬜</t>
         </is>
       </c>
     </row>
-    <row r="100" hidden="1">
+    <row r="100">
       <c r="A100" s="16" t="n"/>
       <c r="B100" s="28" t="n">
         <v>99</v>
@@ -4020,40 +4032,44 @@
         </is>
       </c>
     </row>
-    <row r="101" hidden="1">
+    <row r="101">
       <c r="A101" s="16" t="n"/>
-      <c r="B101" s="28" t="n">
+      <c r="B101" s="32" t="n">
         <v>100</v>
       </c>
-      <c r="C101" s="28" t="inlineStr">
+      <c r="C101" s="32" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D101" s="29" t="inlineStr">
+      <c r="D101" s="33" t="inlineStr">
         <is>
           <t>https://meli.la/1c6vAL2</t>
         </is>
       </c>
-      <c r="E101" s="30" t="inlineStr">
+      <c r="E101" s="34" t="inlineStr">
         <is>
           <t>Fone De Ouvido Aberto Indicador De Bateria Ipx7 Para Corrida,fone De Ouvido Bluetooth Com Ear Clip Tws Ows Hifi Esportivo 72h Bateria Ipx7 Prova D'água E Suor Enc Cancelamento Ruído</t>
         </is>
       </c>
-      <c r="F101" s="28" t="n"/>
-      <c r="G101" s="31" t="inlineStr">
+      <c r="F101" s="32" t="n"/>
+      <c r="G101" s="35" t="inlineStr">
         <is>
           <t>Inova Cases</t>
         </is>
       </c>
-      <c r="H101" s="28" t="n"/>
+      <c r="H101" s="32" t="inlineStr">
+        <is>
+          <t>fora do ar</t>
+        </is>
+      </c>
       <c r="I101" t="inlineStr">
         <is>
           <t>⬜</t>
         </is>
       </c>
     </row>
-    <row r="102" hidden="1">
+    <row r="102">
       <c r="A102" s="16" t="n"/>
       <c r="B102" s="28" t="n">
         <v>101</v>
@@ -4086,66 +4102,70 @@
         </is>
       </c>
     </row>
-    <row r="103" hidden="1">
+    <row r="103">
       <c r="A103" s="3" t="n"/>
-      <c r="B103" s="54" t="n">
+      <c r="B103" s="28" t="n">
         <v>102</v>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C103" s="28" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D103" s="4" t="inlineStr">
+      <c r="D103" s="29" t="inlineStr">
         <is>
           <t>https://meli.la/1N2GQcc</t>
         </is>
       </c>
-      <c r="E103" s="6" t="inlineStr">
+      <c r="E103" s="30" t="inlineStr">
         <is>
           <t>Fone De Ouvido Bluetooth Sem Fio Wave Buds 2 JBL JBLWBUDS2BLK Preto</t>
         </is>
       </c>
-      <c r="F103" s="3" t="n"/>
-      <c r="G103" s="18" t="inlineStr">
+      <c r="F103" s="28" t="n"/>
+      <c r="G103" s="31" t="inlineStr">
         <is>
           <t>JBL</t>
         </is>
       </c>
-      <c r="H103" s="3" t="n"/>
+      <c r="H103" s="28" t="n"/>
       <c r="I103" s="3" t="inlineStr">
         <is>
           <t>⬜</t>
         </is>
       </c>
     </row>
-    <row r="104" hidden="1">
+    <row r="104">
       <c r="A104" s="16" t="n"/>
-      <c r="B104" s="28" t="n">
+      <c r="B104" s="32" t="n">
         <v>103</v>
       </c>
-      <c r="C104" s="28" t="inlineStr">
+      <c r="C104" s="32" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D104" s="29" t="inlineStr">
+      <c r="D104" s="33" t="inlineStr">
         <is>
           <t>https://meli.la/2wA6HkN</t>
         </is>
       </c>
-      <c r="E104" s="30" t="inlineStr">
+      <c r="E104" s="34" t="inlineStr">
         <is>
           <t>Basike Fone De Ouvido Sem Fio Esportivo Bluetooth5.4 TWS, Corrida Gancho, à prova d'água, Com Gan, Tela LED Dupla, Suporta chamadas de voz, adequadas para Android e IOS, Cor Branco</t>
         </is>
       </c>
-      <c r="F104" s="28" t="n"/>
-      <c r="G104" s="31" t="inlineStr">
+      <c r="F104" s="32" t="n"/>
+      <c r="G104" s="35" t="inlineStr">
         <is>
           <t>Basike</t>
         </is>
       </c>
-      <c r="H104" s="28" t="n"/>
+      <c r="H104" s="32" t="inlineStr">
+        <is>
+          <t>fora do ar</t>
+        </is>
+      </c>
       <c r="I104" t="inlineStr">
         <is>
           <t>⬜</t>
@@ -7129,28 +7149,32 @@
       <c r="Z190" s="5" t="n"/>
       <c r="AA190" s="5" t="n"/>
     </row>
-    <row r="191" hidden="1">
-      <c r="B191" s="28" t="n">
+    <row r="191">
+      <c r="B191" s="32" t="n">
         <v>190</v>
       </c>
-      <c r="C191" s="28" t="inlineStr">
+      <c r="C191" s="32" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D191" s="40" t="inlineStr">
+      <c r="D191" s="45" t="inlineStr">
         <is>
           <t>https://meli.la/2cGbTdT</t>
         </is>
       </c>
-      <c r="E191" s="30" t="inlineStr">
+      <c r="E191" s="34" t="inlineStr">
         <is>
           <t>Fone Bluetooth 5.3 Tws Sem Fio Anti Ruido A Prova Dagua Compatível Iphone 7 8 X Xr 11 12 13 14 15 16 17 Xs Pro Max Plus Samsung S20 S23 S24 Xiaomi Motorola Android Prova DAgua Wireless Premium</t>
         </is>
       </c>
-      <c r="F191" s="30" t="n"/>
-      <c r="G191" s="30" t="n"/>
-      <c r="H191" s="30" t="n"/>
+      <c r="F191" s="34" t="n"/>
+      <c r="G191" s="34" t="n"/>
+      <c r="H191" s="34" t="inlineStr">
+        <is>
+          <t>fora do ar</t>
+        </is>
+      </c>
       <c r="I191" s="5" t="n"/>
       <c r="J191" s="5" t="n"/>
       <c r="K191" s="5" t="n"/>
@@ -7171,7 +7195,7 @@
       <c r="Z191" s="5" t="n"/>
       <c r="AA191" s="5" t="n"/>
     </row>
-    <row r="192" hidden="1">
+    <row r="192">
       <c r="B192" s="28" t="n">
         <v>191</v>
       </c>
@@ -7212,7 +7236,7 @@
       <c r="Z192" s="5" t="n"/>
       <c r="AA192" s="5" t="n"/>
     </row>
-    <row r="193" hidden="1">
+    <row r="193">
       <c r="B193" s="28" t="n">
         <v>192</v>
       </c>
@@ -7235,34 +7259,34 @@
       <c r="G193" s="28" t="n"/>
       <c r="H193" s="28" t="n"/>
     </row>
-    <row r="194" hidden="1">
-      <c r="B194" s="55" t="n">
+    <row r="194">
+      <c r="B194" s="28" t="n">
         <v>193</v>
       </c>
-      <c r="C194" s="36" t="inlineStr">
+      <c r="C194" s="28" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D194" s="42" t="inlineStr">
+      <c r="D194" s="40" t="inlineStr">
         <is>
           <t>https://meli.la/2gbZpAz</t>
         </is>
       </c>
-      <c r="E194" s="38" t="inlineStr">
+      <c r="E194" s="30" t="inlineStr">
         <is>
           <t>Fone de Ouvido Ows Bluetooth Design Aberto Kaidi 794 Cor Preto</t>
         </is>
       </c>
-      <c r="F194" s="36" t="n"/>
-      <c r="G194" s="36" t="n"/>
-      <c r="H194" s="36" t="inlineStr">
+      <c r="F194" s="28" t="n"/>
+      <c r="G194" s="28" t="n"/>
+      <c r="H194" s="28" t="inlineStr">
         <is>
           <t>estoque baixo</t>
         </is>
       </c>
     </row>
-    <row r="195" hidden="1">
+    <row r="195">
       <c r="B195" s="28" t="n">
         <v>194</v>
       </c>
@@ -7285,7 +7309,7 @@
       <c r="G195" s="28" t="n"/>
       <c r="H195" s="28" t="n"/>
     </row>
-    <row r="196" hidden="1">
+    <row r="196">
       <c r="B196" s="28" t="n">
         <v>195</v>
       </c>
@@ -7308,7 +7332,7 @@
       <c r="G196" s="28" t="n"/>
       <c r="H196" s="28" t="n"/>
     </row>
-    <row r="197" hidden="1">
+    <row r="197">
       <c r="B197" s="28" t="n">
         <v>196</v>
       </c>
@@ -7331,7 +7355,7 @@
       <c r="G197" s="28" t="n"/>
       <c r="H197" s="28" t="n"/>
     </row>
-    <row r="198" hidden="1">
+    <row r="198">
       <c r="B198" s="28" t="n">
         <v>197</v>
       </c>
@@ -7354,7 +7378,7 @@
       <c r="G198" s="28" t="n"/>
       <c r="H198" s="28" t="n"/>
     </row>
-    <row r="199" hidden="1">
+    <row r="199">
       <c r="B199" s="28" t="n">
         <v>198</v>
       </c>
@@ -7377,78 +7401,86 @@
       <c r="G199" s="28" t="n"/>
       <c r="H199" s="28" t="n"/>
     </row>
-    <row r="200" hidden="1">
-      <c r="B200" s="28" t="n">
+    <row r="200">
+      <c r="B200" s="36" t="n">
         <v>199</v>
       </c>
-      <c r="C200" s="28" t="inlineStr">
+      <c r="C200" s="36" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D200" s="40" t="inlineStr">
+      <c r="D200" s="42" t="inlineStr">
         <is>
           <t>https://meli.la/1jGZwC3</t>
         </is>
       </c>
-      <c r="E200" s="30" t="inlineStr">
+      <c r="E200" s="38" t="inlineStr">
         <is>
           <t>Fone De Ouvido Esportivos Sem Fio Bluetooth Impermeável Ipx6</t>
         </is>
       </c>
-      <c r="F200" s="28" t="n"/>
-      <c r="G200" s="28" t="n"/>
-      <c r="H200" s="28" t="n"/>
-    </row>
-    <row r="201" hidden="1">
-      <c r="B201" s="55" t="n">
+      <c r="F200" s="36" t="n"/>
+      <c r="G200" s="36" t="n"/>
+      <c r="H200" s="36" t="inlineStr">
+        <is>
+          <t>estoque baixo</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="B201" s="28" t="n">
         <v>200</v>
       </c>
-      <c r="C201" s="36" t="inlineStr">
+      <c r="C201" s="28" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D201" s="42" t="inlineStr">
+      <c r="D201" s="40" t="inlineStr">
         <is>
           <t>https://meli.la/2G3uu5c</t>
         </is>
       </c>
-      <c r="E201" s="38" t="inlineStr">
+      <c r="E201" s="30" t="inlineStr">
         <is>
           <t>Fone de Ouvido Eardbud AIWA AWS-EB-04-B Bluetooth IPX4 ANC 26 Horas de bateria</t>
         </is>
       </c>
-      <c r="F201" s="36" t="n"/>
-      <c r="G201" s="36" t="n"/>
-      <c r="H201" s="36" t="inlineStr">
+      <c r="F201" s="28" t="n"/>
+      <c r="G201" s="28" t="n"/>
+      <c r="H201" s="28" t="inlineStr">
         <is>
           <t>estoque baixo</t>
         </is>
       </c>
     </row>
-    <row r="202" hidden="1">
-      <c r="B202" s="28" t="n">
+    <row r="202">
+      <c r="B202" s="32" t="n">
         <v>201</v>
       </c>
-      <c r="C202" s="28" t="inlineStr">
+      <c r="C202" s="32" t="inlineStr">
         <is>
           <t>Fone sem fio (bluetooth)</t>
         </is>
       </c>
-      <c r="D202" s="40" t="inlineStr">
+      <c r="D202" s="45" t="inlineStr">
         <is>
           <t>https://meli.la/1A65TWL</t>
         </is>
       </c>
-      <c r="E202" s="30" t="inlineStr">
+      <c r="E202" s="34" t="inlineStr">
         <is>
           <t>Fone De Ouvido Bluetooth Redmi Buds 6 Play Xiaomi Sem Fio Cor Preto</t>
         </is>
       </c>
-      <c r="F202" s="28" t="n"/>
-      <c r="G202" s="28" t="n"/>
-      <c r="H202" s="28" t="n"/>
+      <c r="F202" s="32" t="n"/>
+      <c r="G202" s="32" t="n"/>
+      <c r="H202" s="32" t="inlineStr">
+        <is>
+          <t>fora do ar</t>
+        </is>
+      </c>
     </row>
     <row r="203" hidden="1">
       <c r="B203" s="54" t="n">
@@ -9735,7 +9767,7 @@
   <autoFilter ref="A1:I253">
     <filterColumn colId="2" hiddenButton="0" showButton="1">
       <filters>
-        <filter val="Teclado sem fio"/>
+        <filter val="Fone sem fio (bluetooth)"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -9952,6 +9984,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId210"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
@@ -9962,7 +9995,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
   </cols>

</xml_diff>